<commit_message>
update the flood report
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\Python Scripts\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E39DA225-20FC-49B3-8642-46529BE56A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667CFB5F-30E3-417B-BC54-9C944185E443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="398">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -1171,9 +1171,6 @@
     <t>Frase completa</t>
   </si>
   <si>
-    <t xml:space="preserve">En las últimas horas se registraron importantes acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 125.4 mm y con un máximo de 100 mm/día. Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores (2.3 metros). </t>
-  </si>
-  <si>
     <t>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 105 mm y con un máximo de 35 mm/día. Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una baja probabilidad de que el nivel supere al máximo registrado los días anteriores (8 metros), pero no se puede descartar en su totalidad.</t>
   </si>
   <si>
@@ -1198,28 +1195,46 @@
     <t>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Uruguay, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en las ciudades de Salto Fray Bentos. está en descenso en la ciudad de . Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores (5m en Paysandú ).</t>
   </si>
   <si>
-    <t>Entre 10.00 y 10.60</t>
-  </si>
-  <si>
-    <t>02 - 03 dic</t>
-  </si>
-  <si>
-    <t>Entre 9.46 y 10.22</t>
-  </si>
-  <si>
-    <t>03 - 05 dic</t>
-  </si>
-  <si>
-    <t>Entre 9.00 y 10.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 24 horas se acumularon 70 mm. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, se espera que el nivel del río Cuareim en Artigas supere la cota de aviso (8.00 m) generando inundaciones en la zona del paseo 7 de setiembre. Dado que el nivel pronosticado esta cerca de la cota de seguridad (10.20 m) no se descarta completamenta esta posibilidad. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Estar atentos a posibles inundaciones locales en la zona del paseo 7 de setiembre. </t>
   </si>
   <si>
-    <t>Se registra incrementos del río Cuareim en Artigas con posibilidad de afectar zona paseo 7 de setiembre</t>
+    <t>Se registra incrementos del río Cuareim en Artigas con baja posibilidad de afectar la zona del paseo 7 de setiembre</t>
+  </si>
+  <si>
+    <t>Menor a 2.0 m</t>
+  </si>
+  <si>
+    <t>17 - 18 Enero</t>
+  </si>
+  <si>
+    <t>18 - 20 Enero</t>
+  </si>
+  <si>
+    <t>Menor a 5.0 m</t>
+  </si>
+  <si>
+    <t>Menor a 3.5 m</t>
+  </si>
+  <si>
+    <t>19 - 21 Enero</t>
+  </si>
+  <si>
+    <t>Menor a 5.9 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 24 horas se acumularon 45.7 mm. Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días, con una baja probabilidad de generarse afectaciones a vivienda en la ciudad de Durazno. </t>
+  </si>
+  <si>
+    <t>Entre 8.20 a 8.50 m</t>
+  </si>
+  <si>
+    <t>Entre 6.30 a 6.70 m</t>
+  </si>
+  <si>
+    <t>18 - 19 Enero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 24 horas se acumularon 55.5 mm. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días, el cual se estima que llegue a un nivel entre 6.30 a 6.70 metros y con una bjaa probabilidad de generarse inundaciones en la zona del paseo 7 de setiembre  </t>
   </si>
 </sst>
 </file>
@@ -1751,9 +1766,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1791,7 +1806,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1897,7 +1912,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2039,7 +2054,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2077,7 +2092,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="41">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2089,7 +2104,7 @@
       </c>
       <c r="C3" s="42">
         <f ca="1">TODAY()</f>
-        <v>45262</v>
+        <v>45308</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2101,7 +2116,7 @@
       </c>
       <c r="C4" s="43">
         <f ca="1">$C$3-1</f>
-        <v>45261</v>
+        <v>45307</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2113,7 +2128,7 @@
       </c>
       <c r="C5" s="42">
         <f ca="1">$C$3-2</f>
-        <v>45260</v>
+        <v>45306</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2125,7 +2140,7 @@
       </c>
       <c r="C6" s="43">
         <f ca="1">$C$3+1</f>
-        <v>45263</v>
+        <v>45309</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2137,7 +2152,7 @@
       </c>
       <c r="C7" s="44">
         <f ca="1">$C$3+2</f>
-        <v>45264</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2149,7 +2164,7 @@
       </c>
       <c r="C8" s="42">
         <f ca="1">$C$3+3</f>
-        <v>45265</v>
+        <v>45311</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2160,7 +2175,7 @@
         <v>174</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -2199,7 +2214,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="8">
-        <v>6.1</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2210,7 +2225,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="6">
-        <v>6.9</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2222,7 +2237,7 @@
       </c>
       <c r="C4" s="32">
         <f>IFERROR(ROUND(ABS(C2-C3)*100,0),"-")</f>
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2234,7 +2249,7 @@
       </c>
       <c r="C5" s="39" t="str">
         <f>IFERROR(IF(C4=0,"Permanece",IF(SIGN(C4)=1,"Sube","Baja")),"-")</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2245,7 +2260,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="8">
-        <v>5.4</v>
+        <v>2.0499999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2256,7 +2271,7 @@
         <v>7</v>
       </c>
       <c r="C7" s="6">
-        <v>5.2</v>
+        <v>2.0499999999999998</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2279,7 +2294,7 @@
       </c>
       <c r="C9" s="32">
         <f>IF((C6-C7)&gt;=0,ROUND((C6-C7)*100,0),"")</f>
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2291,7 +2306,7 @@
       </c>
       <c r="C10" s="39" t="str">
         <f>IF(C9=0,"Permanece",IF(C9="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2302,7 +2317,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="8">
-        <v>2.1</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2313,7 +2328,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="6">
-        <v>1.9</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2336,7 +2351,7 @@
       </c>
       <c r="C14" s="32">
         <f>IF((C11-C12)&gt;=0,ROUND((C11-C12)*100,0),"")</f>
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2348,7 +2363,7 @@
       </c>
       <c r="C15" s="39" t="str">
         <f>IF(C14=0,"Permanece",IF(C14="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2358,9 +2373,7 @@
       <c r="B16" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="6">
-        <v>2.6</v>
-      </c>
+      <c r="C16" s="6"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="27" t="s">
@@ -2369,9 +2382,7 @@
       <c r="B17" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="6">
-        <v>2.4</v>
-      </c>
+      <c r="C17" s="6"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
@@ -2393,7 +2404,7 @@
       </c>
       <c r="C19" s="32">
         <f>IF((C16-C17)&gt;=0,ROUND((C16-C17)*100,0),"")</f>
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2405,7 +2416,7 @@
       </c>
       <c r="C20" s="39" t="str">
         <f>IF(C19=0,"Permanece",IF(C19="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2416,7 +2427,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="8">
-        <v>20.399999999999999</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2427,7 +2438,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="6">
-        <v>100</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -2438,7 +2449,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="6">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2449,7 +2460,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="6">
-        <v>30</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -2460,7 +2471,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="6">
-        <v>80</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2471,7 +2482,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="10">
-        <v>65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -2481,8 +2492,8 @@
       <c r="B27" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="11">
-        <v>7.2</v>
+      <c r="C27" s="11" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2493,7 +2504,7 @@
         <v>36</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>40</v>
+        <v>387</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -2503,8 +2514,8 @@
       <c r="B29" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="11">
-        <v>8.9</v>
+      <c r="C29" s="11" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2515,7 +2526,7 @@
         <v>37</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>40</v>
+        <v>388</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2525,8 +2536,8 @@
       <c r="B31" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="11">
-        <v>2.5</v>
+      <c r="C31" s="11" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2537,7 +2548,7 @@
         <v>38</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>40</v>
+        <v>391</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2548,7 +2559,7 @@
         <v>29</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>35</v>
+        <v>392</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2559,7 +2570,7 @@
         <v>39</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>40</v>
+        <v>391</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="198.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2570,7 +2581,7 @@
         <v>41</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>376</v>
+        <v>393</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2638,7 +2649,7 @@
         <v>85</v>
       </c>
       <c r="C2" s="6">
-        <v>5.95</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2649,7 +2660,7 @@
         <v>86</v>
       </c>
       <c r="C3" s="6">
-        <v>5.59</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2670,9 +2681,9 @@
       <c r="B5" s="31" t="s">
         <v>87</v>
       </c>
-      <c r="C5" s="32">
+      <c r="C5" s="32" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>36</v>
+        <v/>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2684,7 +2695,7 @@
       </c>
       <c r="C6" s="39" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2695,7 +2706,7 @@
         <v>91</v>
       </c>
       <c r="C7" s="6">
-        <v>4</v>
+        <v>7.59</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2706,7 +2717,7 @@
         <v>92</v>
       </c>
       <c r="C8" s="6">
-        <v>3.68</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2729,7 +2740,7 @@
       </c>
       <c r="C10" s="32">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>32</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2752,7 +2763,7 @@
         <v>97</v>
       </c>
       <c r="C12" s="6">
-        <v>4.16</v>
+        <v>5.16</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2763,7 +2774,7 @@
         <v>98</v>
       </c>
       <c r="C13" s="6">
-        <v>3.69</v>
+        <v>4.88</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2786,7 +2797,7 @@
       </c>
       <c r="C15" s="32">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>47</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2809,7 +2820,7 @@
         <v>77</v>
       </c>
       <c r="C17" s="8">
-        <v>70</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -2842,7 +2853,7 @@
         <v>80</v>
       </c>
       <c r="C20" s="6">
-        <v>59.5</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2853,7 +2864,7 @@
         <v>81</v>
       </c>
       <c r="C21" s="6">
-        <v>26.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2864,7 +2875,7 @@
         <v>82</v>
       </c>
       <c r="C22" s="10">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -2874,9 +2885,7 @@
       <c r="B23" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>385</v>
-      </c>
+      <c r="C23" s="11"/>
     </row>
     <row r="24" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="29" t="s">
@@ -2885,9 +2894,7 @@
       <c r="B24" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="12" t="s">
-        <v>386</v>
-      </c>
+      <c r="C24" s="12"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="28" t="s">
@@ -2897,7 +2904,7 @@
         <v>95</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2908,7 +2915,7 @@
         <v>96</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -2919,7 +2926,7 @@
         <v>101</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2930,10 +2937,10 @@
         <v>102</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="231.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="215.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="28" t="s">
         <v>67</v>
       </c>
@@ -2941,7 +2948,7 @@
         <v>83</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2952,7 +2959,7 @@
         <v>84</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -3508,7 +3515,7 @@
         <v>121</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3898,7 +3905,7 @@
         <v>180</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3909,7 +3916,7 @@
         <v>175</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3920,7 +3927,7 @@
         <v>176</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -3931,7 +3938,7 @@
         <v>203</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3942,7 +3949,7 @@
         <v>204</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -3953,7 +3960,7 @@
         <v>205</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3964,7 +3971,7 @@
         <v>206</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -3986,7 +3993,7 @@
         <v>210</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="248.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3997,7 +4004,7 @@
         <v>202</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4277,7 +4284,7 @@
         <v>255</v>
       </c>
       <c r="C21" s="72" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4602,13 +4609,13 @@
       </c>
       <c r="F23" s="54" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
-        <v>En las últimas horas se registraron importantes acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 125.4 mm y con un máximo de 100 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 47.7 mm y con un máximo de 45.7 mm/día.</v>
       </c>
       <c r="G23" s="54"/>
       <c r="H23" s="54"/>
       <c r="I23" s="54" t="str">
         <f>_xlfn.CONCAT($F$8,D23,IF(YI!C15=$E$8,$I$8,IF(YI!C15=$E$9,$I$9,$I$10)),$J$8,E23,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno. </v>
       </c>
       <c r="J23" s="54" t="str">
         <f>_xlfn.CONCAT(F13,IF(YI!C31&gt;YI!C11,I13, IF(YI!C31=YI!C11,I14, I15)))</f>
@@ -4620,7 +4627,7 @@
       </c>
       <c r="L23" s="54" t="str">
         <f>+_xlfn.CONCAT(F23," ",I23, " ",J23," ",K23)</f>
-        <v xml:space="preserve">En las últimas horas se registraron importantes acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 125.4 mm y con un máximo de 100 mm/día. Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores (2.3 metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 47.7 mm y con un máximo de 45.7 mm/día. Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores (2.3 metros). </v>
       </c>
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
@@ -4635,7 +4642,7 @@
       </c>
       <c r="F24" s="55" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 70 mm y con un máximo de 70 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 55.5 mm y con un máximo de 55.5 mm/día.</v>
       </c>
       <c r="G24" s="55"/>
       <c r="H24" s="55"/>
@@ -4653,7 +4660,7 @@
       </c>
       <c r="L24" s="54" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 70 mm y con un máximo de 70 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 55.5 mm y con un máximo de 55.5 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
agregar archivos faltantes a la automatizacion qgis
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\Python Scripts\automatic docx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667CFB5F-30E3-417B-BC54-9C944185E443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA368B9-4262-4B8A-A7C0-B20E17C0AF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="C3" s="42">
         <f ca="1">TODAY()</f>
-        <v>45308</v>
+        <v>45338</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="C4" s="43">
         <f ca="1">$C$3-1</f>
-        <v>45307</v>
+        <v>45337</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="C5" s="42">
         <f ca="1">$C$3-2</f>
-        <v>45306</v>
+        <v>45336</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="C6" s="43">
         <f ca="1">$C$3+1</f>
-        <v>45309</v>
+        <v>45339</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="C7" s="44">
         <f ca="1">$C$3+2</f>
-        <v>45310</v>
+        <v>45340</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C8" s="42">
         <f ca="1">$C$3+3</f>
-        <v>45311</v>
+        <v>45341</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -3699,7 +3699,7 @@
         <v>182</v>
       </c>
       <c r="C12" s="74">
-        <v>13.77</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3710,7 +3710,7 @@
         <v>183</v>
       </c>
       <c r="C13" s="73">
-        <v>13.77</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3731,9 +3731,9 @@
       <c r="B15" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="C15" s="32">
+      <c r="C15" s="32" t="str">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="16" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="C16" s="39" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="I26" s="66" t="str">
         <f>IF(AND(URUGUAY!$C$11=$E$8,URUGUAY!$C$16=$E$8,URUGUAY!$C$21=$E$8,URUGUAY!$C$26=$E$8),_xlfn.CONCAT($F$8,$D$26,$I$8,$J$9," ",E26,", ",E27,", ",E28," y ",Tablas!E29,"."),IF(AND(URUGUAY!$C$11=$E$9,URUGUAY!$C$16=$E$9,URUGUAY!$C$21=$E$9,URUGUAY!$C$26=$E$9),_xlfn.CONCAT($F$8,$D$26,$I$9,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),IF(AND(URUGUAY!$C$11=$E$10,URUGUAY!$C$16=$E$10,URUGUAY!$C$21=$E$10,URUGUAY!$C$26=$E$10),_xlfn.CONCAT($F$8,$D$26,$I$10,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),_xlfn.CONCAT($F$8,D26,I27,I28,I29))))</f>
-        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en las ciudades de Salto Fray Bentos. está en descenso en la ciudad de .</v>
+        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en la ciudad de  Fray Bentos; está en descenso en la ciudad de  Salto.</v>
       </c>
       <c r="J26" s="76" t="str">
         <f>_xlfn.CONCAT(F13,IF(AND(URUGUAY!C31&gt;URUGUAY!C7, URUGUAY!C33&gt;URUGUAY!C12, URUGUAY!C35&gt;URUGUAY!C17, URUGUAY!C37&gt;URUGUAY!C22),I13, IF(AND(URUGUAY!C31=URUGUAY!C7, URUGUAY!C33=URUGUAY!C12, URUGUAY!C35=URUGUAY!C17, URUGUAY!C37=URUGUAY!C22),I14, I15)))</f>
@@ -4724,7 +4724,7 @@
       </c>
       <c r="L26" s="76" t="str">
         <f t="shared" si="0"/>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Uruguay, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en las ciudades de Salto Fray Bentos. está en descenso en la ciudad de . Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores (5m en Paysandú ).</v>
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Uruguay, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en la ciudad de  Fray Bentos; está en descenso en la ciudad de  Salto. Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores (5m en Paysandú ).</v>
       </c>
     </row>
     <row r="27" spans="3:13" ht="33" x14ac:dyDescent="0.3">
@@ -4759,15 +4759,15 @@
       <c r="F28" s="75"/>
       <c r="G28" s="60">
         <f>SUM(URUGUAY!$C$11=Tablas!E9, URUGUAY!$C$16=Tablas!E9,URUGUAY!$C$21=Tablas!E9,URUGUAY!$C$26=Tablas!E9)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H28" s="61" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E9,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E9,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E9,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E9,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Salto Fray Bentos</v>
+        <v xml:space="preserve"> Fray Bentos</v>
       </c>
       <c r="I28" s="67" t="str">
         <f>_xlfn.CONCAT(I9,IF(G28&gt;1,$J$9,$J$8),H28, IF((G27+G28)=4,".", ";"))</f>
-        <v xml:space="preserve"> se mantiene constante en las ciudades de Salto Fray Bentos.</v>
+        <v xml:space="preserve"> se mantiene constante en la ciudad de  Fray Bentos;</v>
       </c>
       <c r="J28" s="76"/>
       <c r="K28" s="76"/>
@@ -4782,15 +4782,15 @@
       <c r="F29" s="75"/>
       <c r="G29" s="60">
         <f>SUM(URUGUAY!$C$11=Tablas!E10, URUGUAY!$C$16=Tablas!E10,URUGUAY!$C$21=Tablas!E10,URUGUAY!$C$26=Tablas!E10)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29" s="61" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E10,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E10,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E10,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E10,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v/>
+        <v xml:space="preserve"> Salto</v>
       </c>
       <c r="I29" s="67" t="str">
         <f>_xlfn.CONCAT(I10,IF(G29&gt;1,$J$9,$J$8),H29, ".")</f>
-        <v xml:space="preserve"> está en descenso en la ciudad de .</v>
+        <v xml:space="preserve"> está en descenso en la ciudad de  Salto.</v>
       </c>
       <c r="J29" s="76"/>
       <c r="K29" s="76"/>

</xml_diff>

<commit_message>
update the automatic model routine with newest version
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\Python Scripts\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA368B9-4262-4B8A-A7C0-B20E17C0AF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A650A14E-4E5E-4BC6-9A2A-BBD2F64A0869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="397">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -829,9 +829,6 @@
     <t xml:space="preserve">Estar atentos a los próximos eventos de lluvia que se registren en la cuenca.   </t>
   </si>
   <si>
-    <t xml:space="preserve">Estar atentos a los pronósticos meteorológicos que realiza el INUMET.   </t>
-  </si>
-  <si>
     <t xml:space="preserve">Mantener el monitoreo hidrológico reforzado en la zona y estar atento a las actualizaciones de pronósticos del tiempo para los próximos días. </t>
   </si>
   <si>
@@ -1225,16 +1222,16 @@
     <t xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Yí, donde en las últimas 24 horas se acumularon 45.7 mm. Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días, con una baja probabilidad de generarse afectaciones a vivienda en la ciudad de Durazno. </t>
   </si>
   <si>
-    <t>Entre 8.20 a 8.50 m</t>
-  </si>
-  <si>
-    <t>Entre 6.30 a 6.70 m</t>
-  </si>
-  <si>
     <t>18 - 19 Enero</t>
   </si>
   <si>
-    <t xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 24 horas se acumularon 55.5 mm. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días, el cual se estima que llegue a un nivel entre 6.30 a 6.70 metros y con una bjaa probabilidad de generarse inundaciones en la zona del paseo 7 de setiembre  </t>
+    <t xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 59.6 mm y con un máximo de 49.5 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </t>
+  </si>
+  <si>
+    <t>Entre 7.40 a 7.65 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estar atentos a los pronósticos meteorológicos que realiza el INUMET y a los próximos eventos de lluvia que se registren en la cuenca.   </t>
   </si>
 </sst>
 </file>
@@ -2092,7 +2089,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="41">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2104,7 +2101,7 @@
       </c>
       <c r="C3" s="42">
         <f ca="1">TODAY()</f>
-        <v>45338</v>
+        <v>45342</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2116,7 +2113,7 @@
       </c>
       <c r="C4" s="43">
         <f ca="1">$C$3-1</f>
-        <v>45337</v>
+        <v>45341</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2128,7 +2125,7 @@
       </c>
       <c r="C5" s="42">
         <f ca="1">$C$3-2</f>
-        <v>45336</v>
+        <v>45340</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2140,7 +2137,7 @@
       </c>
       <c r="C6" s="43">
         <f ca="1">$C$3+1</f>
-        <v>45339</v>
+        <v>45343</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2152,7 +2149,7 @@
       </c>
       <c r="C7" s="44">
         <f ca="1">$C$3+2</f>
-        <v>45340</v>
+        <v>45344</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2164,7 +2161,7 @@
       </c>
       <c r="C8" s="42">
         <f ca="1">$C$3+3</f>
-        <v>45341</v>
+        <v>45345</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2175,7 +2172,7 @@
         <v>174</v>
       </c>
       <c r="C9" s="45" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -2276,10 +2273,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
+        <v>350</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>351</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>352</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>257</v>
@@ -2333,10 +2330,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C13" s="6">
         <v>2.2999999999999998</v>
@@ -2386,10 +2383,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="27" t="s">
+        <v>344</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>345</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>346</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>257</v>
@@ -2493,7 +2490,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2504,18 +2501,18 @@
         <v>36</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="28" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2526,7 +2523,7 @@
         <v>37</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2537,7 +2534,7 @@
         <v>28</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2548,7 +2545,7 @@
         <v>38</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2559,7 +2556,7 @@
         <v>29</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2570,7 +2567,7 @@
         <v>39</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="198.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2581,10 +2578,10 @@
         <v>41</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="30" t="s">
         <v>68</v>
       </c>
@@ -2592,7 +2589,7 @@
         <v>43</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -2649,7 +2646,7 @@
         <v>85</v>
       </c>
       <c r="C2" s="6">
-        <v>5.6</v>
+        <v>4.6900000000000004</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2660,15 +2657,15 @@
         <v>86</v>
       </c>
       <c r="C3" s="6">
-        <v>5.75</v>
+        <v>4.71</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
+        <v>344</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>345</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>346</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>257</v>
@@ -2706,7 +2703,7 @@
         <v>91</v>
       </c>
       <c r="C7" s="6">
-        <v>7.59</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2717,15 +2714,15 @@
         <v>92</v>
       </c>
       <c r="C8" s="6">
-        <v>7.1</v>
+        <v>7.21</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
+        <v>346</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>347</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>348</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>257</v>
@@ -2738,9 +2735,9 @@
       <c r="B10" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="C10" s="32">
+      <c r="C10" s="32" t="str">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>49</v>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2752,7 +2749,7 @@
       </c>
       <c r="C11" s="39" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2763,7 +2760,7 @@
         <v>97</v>
       </c>
       <c r="C12" s="6">
-        <v>5.16</v>
+        <v>7.25</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2774,15 +2771,15 @@
         <v>98</v>
       </c>
       <c r="C13" s="6">
-        <v>4.88</v>
+        <v>7.21</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>257</v>
@@ -2797,7 +2794,7 @@
       </c>
       <c r="C15" s="32">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>28</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2820,7 +2817,7 @@
         <v>77</v>
       </c>
       <c r="C17" s="8">
-        <v>55.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -2831,7 +2828,7 @@
         <v>78</v>
       </c>
       <c r="C18" s="6">
-        <v>0</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -2842,7 +2839,7 @@
         <v>79</v>
       </c>
       <c r="C19" s="6">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -2853,7 +2850,7 @@
         <v>80</v>
       </c>
       <c r="C20" s="6">
-        <v>13.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2878,14 +2875,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="28" t="s">
         <v>105</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="11"/>
     </row>
     <row r="24" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="29" t="s">
@@ -2894,7 +2890,7 @@
       <c r="B24" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="12"/>
+      <c r="C24" s="11"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="28" t="s">
@@ -2903,9 +2899,7 @@
       <c r="B25" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C25" s="11" t="s">
-        <v>394</v>
-      </c>
+      <c r="C25" s="11"/>
     </row>
     <row r="26" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="29" t="s">
@@ -2914,9 +2908,7 @@
       <c r="B26" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="C26" s="12" t="s">
-        <v>387</v>
-      </c>
+      <c r="C26" s="12"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="28" t="s">
@@ -2937,10 +2929,10 @@
         <v>102</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="215.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="28" t="s">
         <v>67</v>
       </c>
@@ -2948,7 +2940,7 @@
         <v>83</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2959,7 +2951,7 @@
         <v>84</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -3070,10 +3062,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
+        <v>334</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>335</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>336</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>257</v>
@@ -3127,10 +3119,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
+        <v>336</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>337</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>338</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>257</v>
@@ -3184,10 +3176,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>257</v>
@@ -3241,10 +3233,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
+        <v>340</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>341</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>342</v>
       </c>
       <c r="C19" s="6">
         <v>8</v>
@@ -3298,10 +3290,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
+        <v>342</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>343</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>344</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>257</v>
@@ -3515,7 +3507,7 @@
         <v>121</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3526,7 +3518,7 @@
         <v>122</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -3599,10 +3591,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
+        <v>322</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>323</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>324</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>257</v>
@@ -3657,10 +3649,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
+        <v>324</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>325</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>326</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>257</v>
@@ -3699,7 +3691,7 @@
         <v>182</v>
       </c>
       <c r="C12" s="74">
-        <v>7</v>
+        <v>13.77</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3710,15 +3702,15 @@
         <v>183</v>
       </c>
       <c r="C13" s="73">
-        <v>7.1</v>
+        <v>13.77</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
+        <v>326</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>327</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>328</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>257</v>
@@ -3731,9 +3723,9 @@
       <c r="B15" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="C15" s="32" t="str">
+      <c r="C15" s="32">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3745,7 +3737,7 @@
       </c>
       <c r="C16" s="39" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3772,10 +3764,10 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="27" t="s">
+        <v>328</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>329</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>330</v>
       </c>
       <c r="C19" s="6">
         <v>5</v>
@@ -3829,10 +3821,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="27" t="s">
+        <v>330</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>331</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>332</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>257</v>
@@ -3905,7 +3897,7 @@
         <v>180</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3916,7 +3908,7 @@
         <v>175</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3927,7 +3919,7 @@
         <v>176</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -3938,7 +3930,7 @@
         <v>203</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3949,7 +3941,7 @@
         <v>204</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -3960,7 +3952,7 @@
         <v>205</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3971,7 +3963,7 @@
         <v>206</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -3993,7 +3985,7 @@
         <v>210</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="248.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4004,7 +3996,7 @@
         <v>202</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4015,7 +4007,7 @@
         <v>227</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -4087,10 +4079,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
+        <v>332</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>333</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>334</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>257</v>
@@ -4144,10 +4136,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>257</v>
@@ -4284,7 +4276,7 @@
         <v>255</v>
       </c>
       <c r="C21" s="72" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4326,7 +4318,7 @@
   <dimension ref="A1:M30"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="128.42578125" style="47" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="140.85546875" style="47" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="11.42578125" style="47"/>
     <col min="4" max="4" width="14.85546875" style="47" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.28515625" style="47" bestFit="1" customWidth="1"/>
@@ -4345,7 +4337,7 @@
         <v>260</v>
       </c>
       <c r="C1" s="46" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D1" s="51"/>
       <c r="E1" s="51"/>
@@ -4363,26 +4355,26 @@
         <v>261</v>
       </c>
       <c r="C2" s="49" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D2" s="49" t="s">
+        <v>275</v>
+      </c>
+      <c r="E2" s="49" t="s">
         <v>276</v>
       </c>
-      <c r="E2" s="49" t="s">
-        <v>277</v>
-      </c>
       <c r="F2" s="50" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="G2" s="56"/>
       <c r="H2" s="56"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="47" t="s">
-        <v>262</v>
+        <v>396</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D3" s="47">
         <v>70</v>
@@ -4391,24 +4383,24 @@
         <v>200</v>
       </c>
       <c r="F3" s="47" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="I3" s="47" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J3" s="47" t="s">
+        <v>269</v>
+      </c>
+      <c r="K3" s="47" t="s">
         <v>270</v>
-      </c>
-      <c r="K3" s="47" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="47" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D4" s="47">
         <v>30</v>
@@ -4417,20 +4409,20 @@
         <v>100</v>
       </c>
       <c r="F4" s="47" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="47" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F5" s="47" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="47" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -4438,10 +4430,10 @@
         <v>42</v>
       </c>
       <c r="E7" s="49" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F7" s="48" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G7" s="48"/>
       <c r="H7" s="48"/>
@@ -4453,49 +4445,49 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E8" s="47" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F8" s="47" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="I8" s="47" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J8" s="47" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E9" s="47" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="I9" s="47" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J9" s="47" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E10" s="47" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I10" s="47" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C12" s="49" t="s">
+        <v>280</v>
+      </c>
+      <c r="D12" s="49" t="s">
+        <v>278</v>
+      </c>
+      <c r="E12" s="49" t="s">
         <v>281</v>
       </c>
-      <c r="D12" s="49" t="s">
-        <v>279</v>
-      </c>
-      <c r="E12" s="49" t="s">
-        <v>282</v>
-      </c>
       <c r="F12" s="48" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G12" s="48"/>
       <c r="H12" s="48"/>
@@ -4507,43 +4499,43 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D13" s="47" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F13" s="47" t="s">
+        <v>366</v>
+      </c>
+      <c r="I13" s="47" t="s">
         <v>367</v>
-      </c>
-      <c r="I13" s="47" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D14" s="47" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="I14" s="47" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D15" s="47" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I15" s="47" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="49" t="s">
+        <v>280</v>
+      </c>
+      <c r="D17" s="49" t="s">
+        <v>278</v>
+      </c>
+      <c r="E17" s="49" t="s">
         <v>281</v>
       </c>
-      <c r="D17" s="49" t="s">
-        <v>279</v>
-      </c>
-      <c r="E17" s="49" t="s">
-        <v>282</v>
-      </c>
       <c r="F17" s="48" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G17" s="48"/>
       <c r="H17" s="48"/>
@@ -4555,57 +4547,57 @@
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="F18" s="47" t="s">
+        <v>271</v>
+      </c>
+      <c r="I18" s="47" t="s">
         <v>272</v>
-      </c>
-      <c r="I18" s="47" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="F19" s="47" t="s">
+        <v>273</v>
+      </c>
+      <c r="I19" s="47" t="s">
         <v>274</v>
-      </c>
-      <c r="I19" s="47" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="52" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D22" s="52" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E22" s="52" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F22" s="52" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G22" s="52"/>
       <c r="H22" s="52"/>
       <c r="I22" s="52" t="s">
+        <v>309</v>
+      </c>
+      <c r="J22" s="52" t="s">
         <v>310</v>
       </c>
-      <c r="J22" s="52" t="s">
+      <c r="K22" s="52" t="s">
         <v>311</v>
       </c>
-      <c r="K22" s="52" t="s">
-        <v>312</v>
-      </c>
       <c r="L22" s="71" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="23" spans="3:13" s="65" customFormat="1" ht="99" x14ac:dyDescent="0.25">
       <c r="C23" s="65" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D23" s="65" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E23" s="65" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F23" s="54" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
@@ -4632,17 +4624,17 @@
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
       <c r="C24" s="53" t="s">
+        <v>298</v>
+      </c>
+      <c r="D24" s="53" t="s">
         <v>299</v>
       </c>
-      <c r="D24" s="53" t="s">
-        <v>300</v>
-      </c>
       <c r="E24" s="53" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F24" s="55" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 55.5 mm y con un máximo de 55.5 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 59.6 mm y con un máximo de 49.5 mm/día.</v>
       </c>
       <c r="G24" s="55"/>
       <c r="H24" s="55"/>
@@ -4660,18 +4652,18 @@
       </c>
       <c r="L24" s="54" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 55.5 mm y con un máximo de 55.5 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 59.6 mm y con un máximo de 49.5 mm/día. Actualmente, el nivel del río Cuareim está en ascenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">
       <c r="C25" s="53" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D25" s="53" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E25" s="53" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F25" s="54" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(SANTALUCIA!C27:C29)&gt;$D$3,SUM(SANTALUCIA!C27:C29)&gt;$E$3),$F$3,IF(OR(MAX(SANTALUCIA!C27:C29)&gt;$D$4,SUM(SANTALUCIA!C27:C29)&gt;$E$4),$F$4,$F$5)),D25,$I$3,SUM(SANTALUCIA!C27:C29),$J$3,MAX(SANTALUCIA!C27:C29),$K$3)</f>
@@ -4698,13 +4690,13 @@
     </row>
     <row r="26" spans="3:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C26" s="53" t="s">
+        <v>301</v>
+      </c>
+      <c r="D26" s="53" t="s">
         <v>302</v>
       </c>
-      <c r="D26" s="53" t="s">
+      <c r="E26" s="53" t="s">
         <v>303</v>
-      </c>
-      <c r="E26" s="53" t="s">
-        <v>304</v>
       </c>
       <c r="F26" s="75" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(URUGUAY!C27:C29)&gt;$D$3,SUM(URUGUAY!C27:C29)&gt;$E$3),$F$3,IF(OR(MAX(URUGUAY!C27:C29)&gt;$D$4,SUM(URUGUAY!C27:C29)&gt;$E$4),$F$4,$F$5)),D26,$I$3,SUM(URUGUAY!C27:C29),$J$3,MAX(URUGUAY!C27:C29),$K$3)</f>
@@ -4712,7 +4704,7 @@
       </c>
       <c r="I26" s="66" t="str">
         <f>IF(AND(URUGUAY!$C$11=$E$8,URUGUAY!$C$16=$E$8,URUGUAY!$C$21=$E$8,URUGUAY!$C$26=$E$8),_xlfn.CONCAT($F$8,$D$26,$I$8,$J$9," ",E26,", ",E27,", ",E28," y ",Tablas!E29,"."),IF(AND(URUGUAY!$C$11=$E$9,URUGUAY!$C$16=$E$9,URUGUAY!$C$21=$E$9,URUGUAY!$C$26=$E$9),_xlfn.CONCAT($F$8,$D$26,$I$9,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),IF(AND(URUGUAY!$C$11=$E$10,URUGUAY!$C$16=$E$10,URUGUAY!$C$21=$E$10,URUGUAY!$C$26=$E$10),_xlfn.CONCAT($F$8,$D$26,$I$10,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),_xlfn.CONCAT($F$8,D26,I27,I28,I29))))</f>
-        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en la ciudad de  Fray Bentos; está en descenso en la ciudad de  Salto.</v>
+        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en las ciudades de Salto Fray Bentos. está en descenso en la ciudad de .</v>
       </c>
       <c r="J26" s="76" t="str">
         <f>_xlfn.CONCAT(F13,IF(AND(URUGUAY!C31&gt;URUGUAY!C7, URUGUAY!C33&gt;URUGUAY!C12, URUGUAY!C35&gt;URUGUAY!C17, URUGUAY!C37&gt;URUGUAY!C22),I13, IF(AND(URUGUAY!C31=URUGUAY!C7, URUGUAY!C33=URUGUAY!C12, URUGUAY!C35=URUGUAY!C17, URUGUAY!C37=URUGUAY!C22),I14, I15)))</f>
@@ -4724,14 +4716,14 @@
       </c>
       <c r="L26" s="76" t="str">
         <f t="shared" si="0"/>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Uruguay, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en la ciudad de  Fray Bentos; está en descenso en la ciudad de  Salto. Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores (5m en Paysandú ).</v>
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Uruguay, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Paysandú; se mantiene constante en las ciudades de Salto Fray Bentos. está en descenso en la ciudad de . Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores (5m en Paysandú ).</v>
       </c>
     </row>
     <row r="27" spans="3:13" ht="33" x14ac:dyDescent="0.3">
       <c r="C27" s="53"/>
       <c r="D27" s="53"/>
       <c r="E27" s="53" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F27" s="75"/>
       <c r="G27" s="60">
@@ -4754,20 +4746,20 @@
       <c r="C28" s="53"/>
       <c r="D28" s="53"/>
       <c r="E28" s="53" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F28" s="75"/>
       <c r="G28" s="60">
         <f>SUM(URUGUAY!$C$11=Tablas!E9, URUGUAY!$C$16=Tablas!E9,URUGUAY!$C$21=Tablas!E9,URUGUAY!$C$26=Tablas!E9)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28" s="61" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E9,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E9,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E9,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E9,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Fray Bentos</v>
+        <v xml:space="preserve"> Salto Fray Bentos</v>
       </c>
       <c r="I28" s="67" t="str">
         <f>_xlfn.CONCAT(I9,IF(G28&gt;1,$J$9,$J$8),H28, IF((G27+G28)=4,".", ";"))</f>
-        <v xml:space="preserve"> se mantiene constante en la ciudad de  Fray Bentos;</v>
+        <v xml:space="preserve"> se mantiene constante en las ciudades de Salto Fray Bentos.</v>
       </c>
       <c r="J28" s="76"/>
       <c r="K28" s="76"/>
@@ -4777,20 +4769,20 @@
       <c r="C29" s="53"/>
       <c r="D29" s="53"/>
       <c r="E29" s="53" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F29" s="75"/>
       <c r="G29" s="60">
         <f>SUM(URUGUAY!$C$11=Tablas!E10, URUGUAY!$C$16=Tablas!E10,URUGUAY!$C$21=Tablas!E10,URUGUAY!$C$26=Tablas!E10)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" s="61" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E10,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E10,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E10,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E10,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Salto</v>
+        <v/>
       </c>
       <c r="I29" s="67" t="str">
         <f>_xlfn.CONCAT(I10,IF(G29&gt;1,$J$9,$J$8),H29, ".")</f>
-        <v xml:space="preserve"> está en descenso en la ciudad de  Salto.</v>
+        <v xml:space="preserve"> está en descenso en la ciudad de .</v>
       </c>
       <c r="J29" s="76"/>
       <c r="K29" s="76"/>
@@ -4798,13 +4790,13 @@
     </row>
     <row r="30" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
       <c r="C30" s="53" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D30" s="53" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E30" s="53" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F30" s="54" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(NEGRO!C12:C14)&gt;$D$3,SUM(NEGRO!C12:C14)&gt;$E$3),$F$3,IF(OR(MAX(NEGRO!C12:C14)&gt;$D$4,SUM(NEGRO!C12:C14)&gt;$E$4),$F$4,$F$5)),D30,$I$3,SUM(NEGRO!C12:C14),$J$3,MAX(NEGRO!C12:C14),$K$3)</f>
@@ -4857,16 +4849,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="59" t="s">
+        <v>354</v>
+      </c>
+      <c r="B1" s="59" t="s">
         <v>355</v>
       </c>
-      <c r="B1" s="59" t="s">
+      <c r="C1" s="62" t="s">
         <v>356</v>
       </c>
-      <c r="C1" s="62" t="s">
-        <v>357</v>
-      </c>
       <c r="D1" s="62" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -4874,13 +4866,13 @@
         <v>45224</v>
       </c>
       <c r="B2" t="s">
+        <v>357</v>
+      </c>
+      <c r="C2" s="63" t="s">
         <v>358</v>
       </c>
-      <c r="C2" s="63" t="s">
-        <v>359</v>
-      </c>
       <c r="D2" s="63" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -4888,10 +4880,10 @@
         <v>45224</v>
       </c>
       <c r="B3" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C3" s="63" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -4899,13 +4891,13 @@
         <v>45224</v>
       </c>
       <c r="B4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C4" s="63" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D4" s="63" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -4913,10 +4905,10 @@
         <v>45224</v>
       </c>
       <c r="B5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C5" s="63" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -4924,10 +4916,10 @@
         <v>45224</v>
       </c>
       <c r="B6" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D6" s="64" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -4935,13 +4927,13 @@
         <v>45224</v>
       </c>
       <c r="B7" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C7" s="63" t="s">
+        <v>372</v>
+      </c>
+      <c r="D7" s="63" t="s">
         <v>373</v>
-      </c>
-      <c r="D7" s="63" t="s">
-        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update repository with data march
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C68228-CE5D-4143-B738-B962F6E4D4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5650F14-8FBA-431C-B75C-9E320B008AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="442">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -1287,30 +1287,6 @@
     <t>Menor a 4 metros</t>
   </si>
   <si>
-    <t>Entre 28 y 29 mayo</t>
-  </si>
-  <si>
-    <t>Entre 29 y 30 mayo</t>
-  </si>
-  <si>
-    <t>Entre 30 y 31 mayo</t>
-  </si>
-  <si>
-    <t>Entre 6.90 a 7.80 metros</t>
-  </si>
-  <si>
-    <t>Entre 6.20 a 6.90 metros</t>
-  </si>
-  <si>
-    <t>Menor a 7.60 metros</t>
-  </si>
-  <si>
-    <t>Entre las 07 horas 26 mayo hasta 07 horas 27 de mayo de 2025, en la cuenca del río Yí hasta la ciudad de Durazno se registraron 20 mm en promedio. Actualmente se observa un incremento de nivel del río Yí en Durazno. Algunos modelos de pronóstico de lluvia, indican la posibilidad de lluvia en la cuenca este día. Si las lluvias se cumplen, el escenario mas pesimista es que el nivel del río llegaría entre 6.20 a 6.90 metros el 30 mayo 2025, con lo que se podria generar inundaciones en zona de camping. Inumet comenta que la posibilidad de darse esta precipitación en la cuenca es muy baja.</t>
-  </si>
-  <si>
-    <t>Estar atentos a los acumulados de lluvia en las próximas 24 horas</t>
-  </si>
-  <si>
     <t>Menor a 5 metros</t>
   </si>
   <si>
@@ -1350,12 +1326,6 @@
     <t>Entre 5.50 y 6.10 metros</t>
   </si>
   <si>
-    <t>El río Uruguay se mantiene en ascenso mientras que se registra el descenso del nivel del río Cuareim en Artigas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El río Cuareim en Artigas se encuentra en descenso. El día de ayer en la tarde-noche se registró el nivel máximo de 10.17 metros, estando levemente por debajo de la cota de seguridad (10.20 m) definido para la ciudad. Actualmente se mantiene inundada la zona del paseo 7 de setiembre y el estadio Matias Gonzalez, pero se espera que el día de mañana el río regrese a su cauce. </t>
-  </si>
-  <si>
     <t>12000 y 13500</t>
   </si>
   <si>
@@ -1366,6 +1336,39 @@
   </si>
   <si>
     <t xml:space="preserve">Se mantiene en ascenso el nivel del río Uruguay. CTM-Salto Grande reporta en su comunicado diario que el caudal medio diario evacuado variará entre12000 y 13500 m3/s y la cota máxima y minima en Salto variará entre 8.50 y 9.70 metros. En Paysandú, el nivel del río se mantiene en ascenso y se espera que el río pueda alcanzar los 5 metros, lo cual indica que estaria por debajo de su cota de seguridad (6 metros). En relación a los ríos Daymán y Arapey se encuentran en descenso, mientras que el río Queguay se mantiene en ascenso y en una cota de 5.36 metros. </t>
+  </si>
+  <si>
+    <t>08 Abril</t>
+  </si>
+  <si>
+    <t>09 y 10 abril</t>
+  </si>
+  <si>
+    <t>Entre 10 y 11 abril</t>
+  </si>
+  <si>
+    <t>Menor a 4.50 m</t>
+  </si>
+  <si>
+    <t>Menor a 4.00 m</t>
+  </si>
+  <si>
+    <t>Menor a 8.5 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El río Cuareim se encuentra en descenso </t>
+  </si>
+  <si>
+    <t>Menor a 2.50 m</t>
+  </si>
+  <si>
+    <t>Menor a 3.00 m</t>
+  </si>
+  <si>
+    <t>En las ultimas horas se han registrado incrementos de nivel del río Yí en las localidades de Sarandí del Yí y Polanco del Yí. En la ciudad de Durazno se observó un incremento del caudal del río, el cual permanece en un nivel entorno a los 0.85 m en Puente Viejo. Con este escenario actual se espera que siga el ascenso el nivel del río, sin embargo no se espera que alcance la cota de aviso los próximos días.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durante las últimas horas se registró el nivel máximo del río Cuareim en Artigas el cual alcanzó los 6.14 metros, sin acercarse a la cota de aviso (8.00 m). Actualmente el nivel del río se encuentra en descenso y no se espera nuevo incrementos en los próximos días. </t>
   </si>
 </sst>
 </file>
@@ -2232,7 +2235,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="40">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2244,7 +2247,7 @@
       </c>
       <c r="C3" s="41">
         <f ca="1">TODAY()</f>
-        <v>45807</v>
+        <v>46121</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2256,7 +2259,7 @@
       </c>
       <c r="C4" s="42">
         <f ca="1">$C$3-1</f>
-        <v>45806</v>
+        <v>46120</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2268,7 +2271,7 @@
       </c>
       <c r="C5" s="41">
         <f ca="1">$C$3-2</f>
-        <v>45805</v>
+        <v>46119</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2280,7 +2283,7 @@
       </c>
       <c r="C6" s="42">
         <f ca="1">$C$3+1</f>
-        <v>45808</v>
+        <v>46122</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2292,7 +2295,7 @@
       </c>
       <c r="C7" s="43">
         <f ca="1">$C$3+2</f>
-        <v>45809</v>
+        <v>46123</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2304,7 +2307,7 @@
       </c>
       <c r="C8" s="41">
         <f ca="1">$C$3+3</f>
-        <v>45810</v>
+        <v>46124</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2315,7 +2318,7 @@
         <v>172</v>
       </c>
       <c r="C9" s="44" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -2459,7 +2462,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="73">
-        <v>1.27</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2470,7 +2473,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="72">
-        <v>1.27</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2482,7 +2485,7 @@
       </c>
       <c r="C4" s="31">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2494,7 +2497,7 @@
       </c>
       <c r="C5" s="38" t="str">
         <f>IF(C4=0,"Permanece",IF(C4="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2505,7 +2508,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="73">
-        <v>2.73</v>
+        <v>2.4700000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2516,7 +2519,7 @@
         <v>7</v>
       </c>
       <c r="C7" s="72">
-        <v>2.7</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2562,7 +2565,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="73">
-        <v>1.34</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2573,7 +2576,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="72">
-        <v>1.27</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2594,7 +2597,7 @@
       </c>
       <c r="C14" s="31">
         <f>IF((C11-C12)&gt;=0,ROUND((C11-C12)*100,0),"")</f>
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2606,7 +2609,7 @@
       </c>
       <c r="C15" s="38" t="str">
         <f>IF(C14=0,"Permanece",IF(C14="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2617,7 +2620,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="72">
-        <v>2.56</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2628,7 +2631,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="72">
-        <v>2.5299999999999998</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -2649,7 +2652,7 @@
       </c>
       <c r="C19" s="31">
         <f>IF((C16-C17)&gt;=0,ROUND((C16-C17)*100,0),"")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2661,7 +2664,7 @@
       </c>
       <c r="C20" s="38" t="str">
         <f>IF(C19=0,"Permanece",IF(C19="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2672,7 +2675,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="75">
-        <v>19.7</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2683,7 +2686,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="76">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -2694,7 +2697,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="76">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2705,7 +2708,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="76">
-        <v>32.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -2727,7 +2730,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="77">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -2738,7 +2741,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>413</v>
+        <v>438</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2749,7 +2752,7 @@
         <v>35</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>414</v>
+        <v>432</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -2760,7 +2763,7 @@
         <v>27</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>419</v>
+        <v>439</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2771,7 +2774,7 @@
         <v>36</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>415</v>
+        <v>433</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2782,7 +2785,7 @@
         <v>28</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>418</v>
+        <v>435</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2793,7 +2796,7 @@
         <v>37</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>416</v>
+        <v>433</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2804,7 +2807,7 @@
         <v>29</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>417</v>
+        <v>434</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2815,10 +2818,10 @@
         <v>38</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="231.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="27" t="s">
         <v>65</v>
       </c>
@@ -2826,7 +2829,7 @@
         <v>39</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>420</v>
+        <v>440</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2837,7 +2840,7 @@
         <v>41</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>421</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -2894,7 +2897,7 @@
         <v>83</v>
       </c>
       <c r="C2" s="6">
-        <v>4.59</v>
+        <v>4.54</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2905,7 +2908,7 @@
         <v>84</v>
       </c>
       <c r="C3" s="6">
-        <v>4.5999999999999996</v>
+        <v>4.54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2926,9 +2929,9 @@
       <c r="B5" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="31" t="str">
+      <c r="C5" s="31">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -2940,7 +2943,7 @@
       </c>
       <c r="C6" s="38" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2951,7 +2954,7 @@
         <v>89</v>
       </c>
       <c r="C7" s="6">
-        <v>4.2300000000000004</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2962,7 +2965,7 @@
         <v>90</v>
       </c>
       <c r="C8" s="6">
-        <v>4.3899999999999997</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3008,7 +3011,7 @@
         <v>95</v>
       </c>
       <c r="C12" s="6">
-        <v>9.5299999999999994</v>
+        <v>5.58</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3019,7 +3022,7 @@
         <v>96</v>
       </c>
       <c r="C13" s="6">
-        <v>9.59</v>
+        <v>5.63</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3076,7 +3079,7 @@
         <v>76</v>
       </c>
       <c r="C18" s="76">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -3087,7 +3090,7 @@
         <v>77</v>
       </c>
       <c r="C19" s="76">
-        <v>39</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -3120,7 +3123,7 @@
         <v>80</v>
       </c>
       <c r="C22" s="77">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3131,7 +3134,7 @@
         <v>87</v>
       </c>
       <c r="C23" s="74" t="s">
-        <v>255</v>
+        <v>408</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3142,7 +3145,7 @@
         <v>88</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>255</v>
+        <v>408</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3153,7 +3156,7 @@
         <v>93</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>255</v>
+        <v>408</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3164,7 +3167,7 @@
         <v>94</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>255</v>
+        <v>408</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -3175,7 +3178,7 @@
         <v>99</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>255</v>
+        <v>436</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3186,10 +3189,10 @@
         <v>100</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27" t="s">
         <v>65</v>
       </c>
@@ -3197,10 +3200,10 @@
         <v>81</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="29" t="s">
         <v>66</v>
       </c>
@@ -3208,7 +3211,7 @@
         <v>82</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>371</v>
+        <v>257</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -3585,7 +3588,7 @@
         <v>394</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3596,7 +3599,7 @@
         <v>395</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -3607,7 +3610,7 @@
         <v>121</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3618,7 +3621,7 @@
         <v>122</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -3629,7 +3632,7 @@
         <v>127</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3640,7 +3643,7 @@
         <v>128</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -3669,7 +3672,7 @@
         <v>129</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3680,7 +3683,7 @@
         <v>130</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -3702,7 +3705,7 @@
         <v>136</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3713,7 +3716,7 @@
         <v>119</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3901,7 +3904,7 @@
         <v>161</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -3923,7 +3926,7 @@
         <v>406</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4313,7 +4316,7 @@
         <v>178</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>437</v>
+        <v>427</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -4324,7 +4327,7 @@
         <v>173</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4344,7 +4347,7 @@
         <v>201</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>438</v>
+        <v>428</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4364,7 +4367,7 @@
         <v>203</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>439</v>
+        <v>429</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4402,7 +4405,7 @@
         <v>200</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>440</v>
+        <v>430</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4616,7 +4619,7 @@
         <v>244</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4627,7 +4630,7 @@
         <v>243</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -4676,7 +4679,7 @@
         <v>253</v>
       </c>
       <c r="C21" s="71" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4866,7 +4869,7 @@
         <v>389</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -4886,7 +4889,7 @@
         <v>390</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -5212,13 +5215,13 @@
       </c>
       <c r="F23" s="53" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 19.7 mm y con un máximo de 19.7 mm/día.</v>
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 34.7 mm y con un máximo de 19 mm/día.</v>
       </c>
       <c r="G23" s="53"/>
       <c r="H23" s="53"/>
       <c r="I23" s="53" t="str">
         <f>_xlfn.CONCAT($F$8,D23,IF(YI!C15=$E$8,$I$8,IF(YI!C15=$E$9,$I$9,$I$10)),$J$8,E23,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno. </v>
       </c>
       <c r="J23" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(YI!C31&gt;YI!C11,I13, IF(YI!C31=YI!C11,I14, I15)))</f>
@@ -5230,7 +5233,7 @@
       </c>
       <c r="L23" s="53" t="str">
         <f>+_xlfn.CONCAT(F23," ",I23, " ",J23," ",K23)</f>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 19.7 mm y con un máximo de 19.7 mm/día. Actualmente, el nivel del río Yí está en ascenso en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 34.7 mm y con un máximo de 19 mm/día. Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
@@ -5245,7 +5248,7 @@
       </c>
       <c r="F24" s="54" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 47 mm y con un máximo de 39 mm/día.</v>
+        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 88 mm y con un máximo de 65 mm/día.</v>
       </c>
       <c r="G24" s="54"/>
       <c r="H24" s="54"/>
@@ -5263,7 +5266,7 @@
       </c>
       <c r="L24" s="53" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 47 mm y con un máximo de 39 mm/día. Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 88 mm y con un máximo de 65 mm/día. Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">
@@ -5330,7 +5333,7 @@
         <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Uruguay, donde en las últimas 72 horas se acumularon 36.4 mm y con un máximo de 31.3 mm/día. Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Salto Paysandú; se mantiene constante en la ciudad de ; está en descenso en la ciudad de  Fray Bentos. Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, se prevé que el nivel descienda en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( -m en Paysandú ).</v>
       </c>
     </row>
-    <row r="27" spans="3:13" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:13" ht="33" x14ac:dyDescent="0.3">
       <c r="C27" s="52"/>
       <c r="D27" s="52"/>
       <c r="E27" s="52" t="s">

</xml_diff>

<commit_message>
update generation of automatic flood forecast report
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5650F14-8FBA-431C-B75C-9E320B008AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E523873F-69BF-4E33-AD00-BCA55854B3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="436">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -570,15 +570,6 @@
     <t>fecha_bellaunion</t>
   </si>
   <si>
-    <t>pobs_24_uruguay</t>
-  </si>
-  <si>
-    <t>pobs_48_uruguay</t>
-  </si>
-  <si>
-    <t>pobs_72_uruguay</t>
-  </si>
-  <si>
     <t>q_erogado_ctm</t>
   </si>
   <si>
@@ -759,15 +750,6 @@
     <t>tendencia_mercedes</t>
   </si>
   <si>
-    <t>pobs_24_negro</t>
-  </si>
-  <si>
-    <t>pobs_48_negro</t>
-  </si>
-  <si>
-    <t>pobs_72_negro</t>
-  </si>
-  <si>
     <t>Caudal erogado previsto en Rincón del Bonete</t>
   </si>
   <si>
@@ -1308,12 +1290,6 @@
     <t>Entre las 07 horas 26 mayo hasta 07 horas 27 mayo 2025, las precipitaciones en la cuenca del río San José fueron cercana a los 14 mm. Se espera que el nivel del río aumente ligeramente pero sin generar inconvenientes en la ciudad de San José</t>
   </si>
   <si>
-    <t>Entre 132 a 254 m3/s</t>
-  </si>
-  <si>
-    <t>Entre 179 a 405 m3/s</t>
-  </si>
-  <si>
     <t>En los últimos días se registraron lluvias en la cuenca del río Tacuarembó Chico, las cuales estuvieron en el entorno de 60 a 70 mm. No se prevé condiciones hidrologicas adversas en el río Negro, aunque no se descarta incrementos de nivel en la subcuenca del río Tacuarembó y Tacuarembó Chico.</t>
   </si>
   <si>
@@ -1326,9 +1302,6 @@
     <t>Entre 5.50 y 6.10 metros</t>
   </si>
   <si>
-    <t>12000 y 13500</t>
-  </si>
-  <si>
     <t>Entre 8.50 y 9.70 metros</t>
   </si>
   <si>
@@ -1369,6 +1342,15 @@
   </si>
   <si>
     <t xml:space="preserve">Durante las últimas horas se registró el nivel máximo del río Cuareim en Artigas el cual alcanzó los 6.14 metros, sin acercarse a la cota de aviso (8.00 m). Actualmente el nivel del río se encuentra en descenso y no se espera nuevo incrementos en los próximos días. </t>
+  </si>
+  <si>
+    <t>2000 y 3000</t>
+  </si>
+  <si>
+    <t>1000 y 2000</t>
+  </si>
+  <si>
+    <t>500 y 1000</t>
   </si>
 </sst>
 </file>
@@ -1664,7 +1646,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1685,9 +1667,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2208,117 +2187,117 @@
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" style="18" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" style="18" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="67" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" style="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" style="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="18"/>
+    <col min="1" max="1" width="31.85546875" style="17" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" style="17" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="67" style="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" style="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" style="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="17"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="21" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="38" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="40">
+      <c r="C2" s="39">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="41">
+      <c r="C3" s="40">
         <f ca="1">TODAY()</f>
-        <v>46121</v>
+        <v>46163</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="42">
+      <c r="C4" s="41">
         <f ca="1">$C$3-1</f>
-        <v>46120</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="41">
+      <c r="C5" s="40">
         <f ca="1">$C$3-2</f>
-        <v>46119</v>
+        <v>46161</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="42">
+      <c r="C6" s="41">
         <f ca="1">$C$3+1</f>
-        <v>46122</v>
+        <v>46164</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="43">
+      <c r="C7" s="42">
         <f ca="1">$C$3+2</f>
-        <v>46123</v>
+        <v>46165</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="41">
+      <c r="C8" s="40">
         <f ca="1">$C$3+3</f>
-        <v>46124</v>
+        <v>46166</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="C9" s="44" t="s">
-        <v>437</v>
+      <c r="C9" s="43" t="s">
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -2333,97 +2312,97 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="94.140625" style="62" customWidth="1"/>
-    <col min="4" max="4" width="78.5703125" style="62" customWidth="1"/>
+    <col min="3" max="3" width="94.140625" style="61" customWidth="1"/>
+    <col min="4" max="4" width="78.5703125" style="61" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="57" t="s">
+        <v>344</v>
+      </c>
+      <c r="B1" s="57" t="s">
+        <v>345</v>
+      </c>
+      <c r="C1" s="60" t="s">
+        <v>346</v>
+      </c>
+      <c r="D1" s="60" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="56">
+        <v>45224</v>
+      </c>
+      <c r="B2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C2" s="61" t="s">
+        <v>348</v>
+      </c>
+      <c r="D2" s="61" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="56">
+        <v>45224</v>
+      </c>
+      <c r="B3" t="s">
+        <v>347</v>
+      </c>
+      <c r="C3" s="61" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="56">
+        <v>45224</v>
+      </c>
+      <c r="B4" t="s">
+        <v>347</v>
+      </c>
+      <c r="C4" s="61" t="s">
         <v>350</v>
       </c>
-      <c r="B1" s="58" t="s">
+      <c r="D4" s="61" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="56">
+        <v>45224</v>
+      </c>
+      <c r="B5" t="s">
+        <v>347</v>
+      </c>
+      <c r="C5" s="61" t="s">
         <v>351</v>
       </c>
-      <c r="C1" s="61" t="s">
-        <v>352</v>
-      </c>
-      <c r="D1" s="61" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="57">
+    </row>
+    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="56">
         <v>45224</v>
       </c>
-      <c r="B2" t="s">
-        <v>353</v>
-      </c>
-      <c r="C2" s="62" t="s">
-        <v>354</v>
-      </c>
-      <c r="D2" s="62" t="s">
+      <c r="B6" t="s">
+        <v>347</v>
+      </c>
+      <c r="D6" s="62" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="57">
+    <row r="7" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="56">
         <v>45224</v>
       </c>
-      <c r="B3" t="s">
-        <v>353</v>
-      </c>
-      <c r="C3" s="62" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="57">
-        <v>45224</v>
-      </c>
-      <c r="B4" t="s">
-        <v>353</v>
-      </c>
-      <c r="C4" s="62" t="s">
-        <v>356</v>
-      </c>
-      <c r="D4" s="62" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="57">
-        <v>45224</v>
-      </c>
-      <c r="B5" t="s">
-        <v>353</v>
-      </c>
-      <c r="C5" s="62" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="57">
-        <v>45224</v>
-      </c>
-      <c r="B6" t="s">
-        <v>353</v>
-      </c>
-      <c r="D6" s="63" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="57">
-        <v>45224</v>
-      </c>
       <c r="B7" t="s">
-        <v>353</v>
-      </c>
-      <c r="C7" s="62" t="s">
-        <v>368</v>
-      </c>
-      <c r="D7" s="62" t="s">
-        <v>369</v>
+        <v>347</v>
+      </c>
+      <c r="C7" s="61" t="s">
+        <v>362</v>
+      </c>
+      <c r="D7" s="61" t="s">
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -2438,7 +2417,7 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" style="15" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" style="14" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" style="5" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="5"/>
   </cols>
@@ -2455,392 +2434,392 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
         <v>74</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="73">
-        <v>1.41</v>
+      <c r="C2" s="72">
+        <v>1.84</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="25" t="s">
         <v>43</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="72">
-        <v>1.4</v>
+      <c r="C3" s="71">
+        <v>1.84</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="31">
+      <c r="C4" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="36" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="38" t="str">
+      <c r="C5" s="37" t="str">
         <f>IF(C4=0,"Permanece",IF(C4="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="26" t="s">
         <v>46</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="73">
-        <v>2.4700000000000002</v>
+      <c r="C6" s="72">
+        <v>2.4500000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="25" t="s">
         <v>47</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="72">
-        <v>2.44</v>
+      <c r="C7" s="71">
+        <v>2.46</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
-        <v>346</v>
+      <c r="A8" s="25" t="s">
+        <v>340</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="30" t="str">
         <f>IF((C6-C7)&gt;=0,ROUND((C6-C7)*100,0),"")</f>
-        <v>3</v>
+        <v/>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="38" t="str">
+      <c r="C10" s="37" t="str">
         <f>IF(C9=0,"Permanece",IF(C9="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="26" t="s">
         <v>48</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="73">
-        <v>0.85</v>
+      <c r="C11" s="72">
+        <v>0.75</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="25" t="s">
         <v>49</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="72">
-        <v>0.85</v>
+      <c r="C12" s="71">
+        <v>0.75</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
-        <v>349</v>
+      <c r="A13" s="25" t="s">
+        <v>343</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="C13" s="6"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="30" t="s">
+      <c r="B14" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="30">
         <f>IF((C11-C12)&gt;=0,ROUND((C11-C12)*100,0),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="37" t="s">
+      <c r="B15" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="38" t="str">
+      <c r="C15" s="37" t="str">
         <f>IF(C14=0,"Permanece",IF(C14="","Baja","Sube"))</f>
         <v>Permanece</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="25" t="s">
         <v>50</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="72">
-        <v>2.35</v>
+      <c r="C16" s="71">
+        <v>2.31</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="25" t="s">
         <v>51</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="72">
-        <v>2.35</v>
+      <c r="C17" s="71">
+        <v>2.31</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="26" t="s">
-        <v>349</v>
+      <c r="A18" s="25" t="s">
+        <v>343</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="C18" s="6"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="30" t="s">
+      <c r="B19" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="31">
+      <c r="C19" s="30">
         <f>IF((C16-C17)&gt;=0,ROUND((C16-C17)*100,0),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="38" t="str">
+      <c r="C20" s="37" t="str">
         <f>IF(C19=0,"Permanece",IF(C19="","Baja","Sube"))</f>
         <v>Permanece</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="27" t="s">
+      <c r="A21" s="26" t="s">
         <v>52</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="75">
-        <v>1.7</v>
+      <c r="C21" s="74">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="26" t="s">
+      <c r="A22" s="25" t="s">
         <v>53</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="76">
-        <v>19</v>
+      <c r="C22" s="75">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="26" t="s">
+      <c r="A23" s="25" t="s">
         <v>54</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="76">
-        <v>14</v>
+      <c r="C23" s="75">
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="26" t="s">
+      <c r="A24" s="25" t="s">
         <v>55</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="76">
+      <c r="C24" s="75">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="26" t="s">
+      <c r="A25" s="25" t="s">
         <v>57</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="75">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="77">
-        <v>6</v>
+      <c r="C26" s="76">
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="26" t="s">
         <v>58</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="10" t="s">
-        <v>438</v>
+      <c r="C27" s="9" t="s">
+        <v>429</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C28" s="11" t="s">
-        <v>432</v>
+      <c r="C28" s="10" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="27" t="s">
-        <v>291</v>
+      <c r="A29" s="26" t="s">
+        <v>285</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="10" t="s">
-        <v>439</v>
+      <c r="C29" s="9" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C30" s="11" t="s">
-        <v>433</v>
+      <c r="C30" s="10" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="27" t="s">
+      <c r="A31" s="26" t="s">
         <v>59</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="10" t="s">
-        <v>435</v>
+      <c r="C31" s="9" t="s">
+        <v>426</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="11" t="s">
-        <v>433</v>
+      <c r="C32" s="10" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="27" t="s">
+      <c r="A33" s="26" t="s">
         <v>60</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="10" t="s">
-        <v>434</v>
+      <c r="C33" s="9" t="s">
+        <v>425</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="28" t="s">
+      <c r="A34" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="11" t="s">
-        <v>433</v>
+      <c r="C34" s="10" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="27" t="s">
+      <c r="A35" s="26" t="s">
         <v>65</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="12" t="s">
-        <v>440</v>
+      <c r="C35" s="11" t="s">
+        <v>431</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C36" s="14" t="s">
-        <v>257</v>
+      <c r="C36" s="13" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -2873,7 +2852,7 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" style="15" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" style="14" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" style="5" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="5"/>
   </cols>
@@ -2890,368 +2869,368 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="25" t="s">
         <v>101</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="6">
-        <v>4.54</v>
+      <c r="C2" s="71">
+        <v>3.93</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="25" t="s">
         <v>102</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="6">
-        <v>4.54</v>
+      <c r="C3" s="71">
+        <v>3.94</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>340</v>
+      <c r="A4" s="25" t="s">
+        <v>334</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="38" t="str">
+      <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="25" t="s">
         <v>110</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C7" s="6">
-        <v>3.63</v>
+      <c r="C7" s="71">
+        <v>0.34</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="25" t="s">
         <v>111</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="6">
-        <v>3.66</v>
+      <c r="C8" s="71">
+        <v>0.34</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="26" t="s">
-        <v>342</v>
+      <c r="A9" s="25" t="s">
+        <v>336</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="C10" s="31" t="str">
+      <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="C11" s="38" t="str">
+      <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="25" t="s">
         <v>106</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C12" s="6">
-        <v>5.58</v>
+      <c r="C12" s="71">
+        <v>1.83</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="25" t="s">
         <v>107</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C13" s="6">
-        <v>5.63</v>
+      <c r="C13" s="71">
+        <v>1.85</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="26" t="s">
-        <v>345</v>
+      <c r="A14" s="25" t="s">
+        <v>339</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="30" t="s">
+      <c r="B15" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="C15" s="31" t="str">
+      <c r="C15" s="30" t="str">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="29" t="s">
         <v>98</v>
       </c>
-      <c r="C16" s="38" t="str">
+      <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
         <v>Baja</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="26" t="s">
         <v>52</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C17" s="75">
+      <c r="C17" s="74">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="25" t="s">
         <v>53</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="76">
-        <v>23</v>
+      <c r="C18" s="75">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="25" t="s">
         <v>54</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="76">
-        <v>65</v>
+      <c r="C19" s="75">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="25" t="s">
         <v>55</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="76">
+      <c r="C20" s="75">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="26" t="s">
+      <c r="A21" s="25" t="s">
         <v>57</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="76">
+      <c r="C21" s="75">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="77">
-        <v>6</v>
+      <c r="C22" s="76">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="27" t="s">
+      <c r="A23" s="26" t="s">
         <v>103</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C23" s="74" t="s">
-        <v>408</v>
+      <c r="C23" s="73" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C24" s="10" t="s">
-        <v>408</v>
+      <c r="C24" s="9" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="27" t="s">
+      <c r="A25" s="26" t="s">
         <v>112</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C25" s="10" t="s">
-        <v>408</v>
+      <c r="C25" s="9" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>408</v>
+      <c r="C26" s="9" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="26" t="s">
         <v>108</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C27" s="10" t="s">
-        <v>436</v>
+      <c r="C27" s="9" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="11" t="s">
-        <v>431</v>
+      <c r="C28" s="10" t="s">
+        <v>422</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="27" t="s">
+      <c r="A29" s="26" t="s">
         <v>65</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="12" t="s">
-        <v>441</v>
+      <c r="C29" s="11" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="29" t="s">
+      <c r="A30" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="C30" s="14" t="s">
-        <v>257</v>
+      <c r="C30" s="13" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="K31" s="46"/>
+      <c r="K31" s="45"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="K32" s="46"/>
+      <c r="K32" s="45"/>
     </row>
     <row r="33" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K33" s="46"/>
+      <c r="K33" s="45"/>
     </row>
     <row r="34" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K34" s="46"/>
+      <c r="K34" s="45"/>
     </row>
     <row r="35" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K35" s="46"/>
+      <c r="K35" s="45"/>
     </row>
     <row r="36" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K36" s="46"/>
+      <c r="K36" s="45"/>
     </row>
     <row r="37" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K37" s="46"/>
+      <c r="K37" s="45"/>
     </row>
     <row r="38" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K38" s="46"/>
+      <c r="K38" s="45"/>
     </row>
     <row r="39" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K39" s="46"/>
+      <c r="K39" s="45"/>
     </row>
     <row r="40" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K40" s="46"/>
+      <c r="K40" s="45"/>
     </row>
     <row r="41" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K41" s="46"/>
+      <c r="K41" s="45"/>
     </row>
     <row r="42" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K42" s="46"/>
+      <c r="K42" s="45"/>
     </row>
     <row r="43" spans="11:11" x14ac:dyDescent="0.3">
-      <c r="K43" s="46"/>
+      <c r="K43" s="45"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3282,7 +3261,7 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" style="15" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" style="14" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" style="5" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="5"/>
   </cols>
@@ -3299,435 +3278,435 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
         <v>145</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="C2" s="8">
-        <v>0.3</v>
+      <c r="C2" s="72">
+        <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="25" t="s">
         <v>146</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="C3" s="6">
-        <v>0.3</v>
+      <c r="C3" s="71">
+        <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>330</v>
+      <c r="A4" s="25" t="s">
+        <v>324</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="36" t="s">
         <v>166</v>
       </c>
-      <c r="C6" s="38" t="str">
+      <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
         <v>Permanece</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="26" t="s">
         <v>149</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="8"/>
+      <c r="C7" s="72"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="25" t="s">
         <v>150</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C8" s="6"/>
+      <c r="C8" s="71"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="26" t="s">
-        <v>332</v>
+      <c r="A9" s="25" t="s">
+        <v>326</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="36" t="s">
         <v>126</v>
       </c>
-      <c r="C11" s="38" t="str">
+      <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
         <v>Permanece</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="26" t="s">
         <v>137</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="C12" s="8">
-        <v>1.48</v>
+      <c r="C12" s="72">
+        <v>1.5</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="25" t="s">
         <v>138</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="C13" s="6">
-        <v>1.48</v>
+      <c r="C13" s="71">
+        <v>1.49</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="26" t="s">
-        <v>336</v>
+      <c r="A14" s="25" t="s">
+        <v>330</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="C14" s="6"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="30" t="s">
+      <c r="B15" s="29" t="s">
         <v>169</v>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="36" t="s">
         <v>170</v>
       </c>
-      <c r="C16" s="38" t="str">
+      <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="25" t="s">
         <v>141</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C17" s="6"/>
+      <c r="C17" s="71"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="25" t="s">
         <v>142</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C18" s="6"/>
+      <c r="C18" s="71"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
-        <v>338</v>
+      <c r="A19" s="25" t="s">
+        <v>332</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C19" s="6"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="29" t="s">
         <v>133</v>
       </c>
-      <c r="C20" s="31">
+      <c r="C20" s="30">
         <f>IFERROR(ROUND(ABS(C17-C18)*100,0),"-")</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="37" t="s">
+      <c r="B21" s="36" t="s">
         <v>134</v>
       </c>
-      <c r="C21" s="38" t="str">
+      <c r="C21" s="37" t="str">
         <f>IFERROR(IF(C20=0,"Permanece",IF(SIGN(C20)=1,"Sube","Baja")),"-")</f>
         <v>Permanece</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="27" t="s">
+      <c r="A22" s="26" t="s">
         <v>52</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C22" s="75">
-        <v>9.8000000000000007</v>
+      <c r="C22" s="74">
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="26" t="s">
+      <c r="A23" s="25" t="s">
         <v>53</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C23" s="76">
+      <c r="C23" s="75">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="C24" s="77">
+      <c r="C24" s="76">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="26" t="s">
+      <c r="A25" s="25" t="s">
         <v>55</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="C25" s="76">
-        <v>32.6</v>
+      <c r="C25" s="75">
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="26" t="s">
+      <c r="A26" s="25" t="s">
         <v>57</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="C26" s="76">
+      <c r="C26" s="75">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="C27" s="77">
+      <c r="C27" s="76">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
-        <v>392</v>
+      <c r="A28" s="26" t="s">
+        <v>386</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>394</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>417</v>
+        <v>388</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="28" t="s">
-        <v>393</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>395</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>415</v>
+      <c r="A29" s="27" t="s">
+        <v>387</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>389</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="27" t="s">
+      <c r="A30" s="26" t="s">
         <v>147</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C30" s="10" t="s">
-        <v>417</v>
+      <c r="C30" s="9" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="C31" s="11" t="s">
-        <v>415</v>
+      <c r="C31" s="10" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="26" t="s">
         <v>151</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="C32" s="10" t="s">
-        <v>417</v>
+      <c r="C32" s="9" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="28" t="s">
+      <c r="A33" s="27" t="s">
         <v>152</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="C33" s="11" t="s">
-        <v>416</v>
+      <c r="C33" s="10" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="26" t="s">
-        <v>396</v>
+      <c r="A34" s="25" t="s">
+        <v>390</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>398</v>
-      </c>
-      <c r="C34" s="10"/>
+        <v>392</v>
+      </c>
+      <c r="C34" s="9"/>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="26" t="s">
-        <v>397</v>
+      <c r="A35" s="25" t="s">
+        <v>391</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="C35" s="11"/>
+        <v>393</v>
+      </c>
+      <c r="C35" s="10"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="27" t="s">
+      <c r="A36" s="26" t="s">
         <v>139</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="C36" s="10" t="s">
-        <v>414</v>
+      <c r="C36" s="9" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="28" t="s">
+      <c r="A37" s="27" t="s">
         <v>140</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="C37" s="11" t="s">
-        <v>416</v>
+      <c r="C37" s="10" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="27" t="s">
+      <c r="A38" s="26" t="s">
         <v>143</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="C38" s="10" t="s">
-        <v>413</v>
+      <c r="C38" s="9" t="s">
+        <v>407</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="28" t="s">
+      <c r="A39" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C39" s="11" t="s">
-        <v>415</v>
+      <c r="C39" s="10" t="s">
+        <v>409</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="27" t="s">
+      <c r="A40" s="26" t="s">
         <v>65</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="C40" s="12" t="s">
-        <v>418</v>
+      <c r="C40" s="11" t="s">
+        <v>412</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="B41" s="13" t="s">
+      <c r="B41" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="C41" s="14" t="s">
-        <v>411</v>
+      <c r="C41" s="13" t="s">
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -3759,7 +3738,7 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" style="15" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" style="14" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" style="5" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="5"/>
   </cols>
@@ -3776,168 +3755,170 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
         <v>153</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="C2" s="8">
-        <v>-999</v>
+      <c r="C2" s="72">
+        <v>0.45</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="25" t="s">
         <v>154</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="C3" s="8"/>
+      <c r="C3" s="72">
+        <v>0.45</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>335</v>
+      <c r="A4" s="25" t="s">
+        <v>329</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="C5" s="31" t="str">
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="36" t="s">
         <v>158</v>
       </c>
-      <c r="C6" s="38" t="str">
+      <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="26" t="s">
         <v>52</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>400</v>
-      </c>
-      <c r="C7" s="75">
-        <v>13.5</v>
+        <v>394</v>
+      </c>
+      <c r="C7" s="74">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="25" t="s">
         <v>53</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="C8" s="76">
+        <v>395</v>
+      </c>
+      <c r="C8" s="75">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>402</v>
-      </c>
-      <c r="C9" s="77">
+      <c r="B9" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="C9" s="76">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="25" t="s">
         <v>55</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="C10" s="76">
-        <v>11</v>
+        <v>397</v>
+      </c>
+      <c r="C10" s="75">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="25" t="s">
         <v>57</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="C11" s="76">
+        <v>398</v>
+      </c>
+      <c r="C11" s="75">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>405</v>
-      </c>
-      <c r="C12" s="77">
+      <c r="B12" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="C12" s="76">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
+      <c r="A13" s="25" t="s">
         <v>159</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>419</v>
+      <c r="C13" s="9" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="26" t="s">
+      <c r="A14" s="25" t="s">
         <v>160</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>410</v>
+      <c r="C14" s="10" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="26" t="s">
         <v>65</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>406</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>420</v>
+        <v>400</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="13" t="s">
-        <v>407</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>371</v>
+      <c r="B16" s="12" t="s">
+        <v>401</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -3965,11 +3946,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2155F922-1445-4239-A643-A9F5E09853DC}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" style="15" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" style="14" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" style="5" customWidth="1"/>
     <col min="4" max="4" width="12" style="5" customWidth="1"/>
     <col min="5" max="16384" width="9.140625" style="5"/>
@@ -3987,436 +3968,403 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
-        <v>186</v>
+      <c r="A2" s="26" t="s">
+        <v>183</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="C2" s="72">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
+        <v>184</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C3" s="71">
+        <v>2.42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="25" t="s">
+        <v>312</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>208</v>
+      </c>
+      <c r="C5" s="30" t="str">
+        <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
+        <v/>
+      </c>
+      <c r="D5" s="55"/>
+    </row>
+    <row r="6" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="36" t="s">
         <v>209</v>
       </c>
-      <c r="C2" s="73">
-        <v>6.22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
-        <v>187</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="C6" s="37" t="str">
+        <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
+        <v>Baja</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
+        <v>181</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="C3" s="72">
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>318</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+      <c r="C7" s="72">
+        <v>2.21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="25" t="s">
+        <v>182</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C8" s="71">
+        <v>2.21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="25" t="s">
+        <v>314</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="30" t="s">
-        <v>211</v>
-      </c>
-      <c r="C5" s="31">
-        <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>2</v>
-      </c>
-      <c r="D5" s="56"/>
-    </row>
-    <row r="6" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="36" t="s">
+      <c r="B10" s="29" t="s">
+        <v>212</v>
+      </c>
+      <c r="C10" s="30">
+        <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="55"/>
+    </row>
+    <row r="11" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="37" t="s">
-        <v>212</v>
-      </c>
-      <c r="C6" s="38" t="str">
-        <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Sube</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>184</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="B11" s="36" t="s">
         <v>213</v>
       </c>
-      <c r="C7" s="73">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
-        <v>185</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="C8" s="72">
-        <v>5.46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="26" t="s">
-        <v>320</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="25" t="s">
+      <c r="C11" s="37" t="str">
+        <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
+        <v>Permanece</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="25" t="s">
+        <v>189</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C12" s="72">
+        <v>2.39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="25" t="s">
+        <v>190</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C13" s="71">
+        <v>2.2400000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="25" t="s">
+        <v>316</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="30" t="s">
-        <v>215</v>
-      </c>
-      <c r="C10" s="31">
-        <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>4</v>
-      </c>
-      <c r="D10" s="56"/>
-    </row>
-    <row r="11" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="36" t="s">
+      <c r="B15" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="C15" s="30">
+        <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="37" t="s">
-        <v>216</v>
-      </c>
-      <c r="C11" s="38" t="str">
-        <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Sube</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="26" t="s">
-        <v>192</v>
-      </c>
-      <c r="B12" s="5" t="s">
+      <c r="B16" s="29" t="s">
         <v>180</v>
       </c>
-      <c r="C12" s="73">
-        <v>9.2899999999999991</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="C13" s="72">
-        <v>9.23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="26" t="s">
-        <v>322</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="C15" s="31">
-        <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="30" t="s">
-        <v>183</v>
-      </c>
-      <c r="C16" s="38" t="str">
+      <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
         <v>Sube</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
-        <v>188</v>
+      <c r="A17" s="26" t="s">
+        <v>185</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C17" s="72">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="25" t="s">
+        <v>186</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="C18" s="71">
+        <v>1.27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>216</v>
+      </c>
+      <c r="C20" s="30">
+        <f>IF((C17-C18)&gt;=0,ROUND((C17-C18)*100,0),"")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" s="36" t="s">
         <v>217</v>
       </c>
-      <c r="C17" s="73">
-        <v>4.01</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="26" t="s">
-        <v>189</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="C18" s="72">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="s">
-        <v>324</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" s="30" t="s">
-        <v>219</v>
-      </c>
-      <c r="C20" s="31">
-        <f>IF((C17-C18)&gt;=0,ROUND((C17-C18)*100,0),"")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="37" t="s">
-        <v>220</v>
-      </c>
-      <c r="C21" s="38" t="str">
+      <c r="C21" s="37" t="str">
         <f>IF(C20=0,"Permanece",IF(C20="","Baja","Sube"))</f>
         <v>Sube</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="27" t="s">
-        <v>190</v>
+      <c r="A22" s="26" t="s">
+        <v>187</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="C22" s="73">
-        <v>2.0499999999999998</v>
+        <v>218</v>
+      </c>
+      <c r="C22" s="72">
+        <v>1.43</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="26" t="s">
-        <v>191</v>
+      <c r="A23" s="25" t="s">
+        <v>188</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="C23" s="72">
-        <v>2.06</v>
+        <v>219</v>
+      </c>
+      <c r="C23" s="71">
+        <v>1.45</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="26" t="s">
-        <v>326</v>
+      <c r="A24" s="25" t="s">
+        <v>320</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="30" t="s">
-        <v>223</v>
-      </c>
-      <c r="C25" s="31" t="str">
+      <c r="B25" s="29" t="s">
+        <v>220</v>
+      </c>
+      <c r="C25" s="30" t="str">
         <f>IF((C22-C23)&gt;=0,ROUND((C22-C23)*100,0),"")</f>
         <v/>
       </c>
-      <c r="D25" s="56"/>
+      <c r="D25" s="55"/>
     </row>
     <row r="26" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="36" t="s">
+      <c r="A26" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="37" t="s">
-        <v>224</v>
-      </c>
-      <c r="C26" s="38" t="str">
+      <c r="B26" s="36" t="s">
+        <v>221</v>
+      </c>
+      <c r="C26" s="37" t="str">
         <f>IF(C25=0,"Permanece",IF(C25="","Baja","Sube"))</f>
         <v>Baja</v>
       </c>
-      <c r="D26" s="56"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="7" t="s">
+      <c r="D26" s="55"/>
+    </row>
+    <row r="27" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C27" s="75">
-        <v>0</v>
+      <c r="C27" s="6" t="s">
+        <v>433</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="C28" s="76">
-        <v>5.0999999999999996</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="C29" s="76">
-        <v>31.3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="27" t="s">
+        <v>192</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C29" s="10"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
         <v>194</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="28" t="s">
+      <c r="B31" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="C31" s="10"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="26" t="s">
         <v>195</v>
       </c>
-      <c r="B32" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="C32" s="11"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B32" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="27" t="s">
         <v>196</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="C33" s="10" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="28" t="s">
+      <c r="C33" s="10"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="C34" s="9"/>
+    </row>
+    <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="27" t="s">
+        <v>203</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="C35" s="10"/>
+    </row>
+    <row r="36" spans="1:3" ht="215.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B34" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="C34" s="11"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="27" t="s">
-        <v>198</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="28" t="s">
-        <v>199</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="C36" s="11"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="27" t="s">
-        <v>205</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="C37" s="10"/>
-    </row>
-    <row r="38" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="28" t="s">
-        <v>206</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="C38" s="11"/>
-    </row>
-    <row r="39" spans="1:3" ht="215.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="C39" s="12" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="29" t="s">
+      <c r="C36" s="11" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="B40" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>412</v>
+      <c r="B37" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -4428,13 +4376,13 @@
           <x14:formula1>
             <xm:f>Tablas!$A$2:$A$7</xm:f>
           </x14:formula1>
-          <xm:sqref>C40</xm:sqref>
+          <xm:sqref>C37</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{20FBE439-E25B-4237-A27D-A3EF44FD31CC}">
           <x14:formula1>
             <xm:f>Tablas!$L$26</xm:f>
           </x14:formula1>
-          <xm:sqref>C39</xm:sqref>
+          <xm:sqref>C36</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4444,11 +4392,11 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7698158D-7CF5-4621-99AA-4EF5CEB60D57}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="58.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" style="15" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" style="14" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" style="5" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="5"/>
   </cols>
@@ -4465,232 +4413,199 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
+        <v>223</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="C2" s="72">
+        <v>9.56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="C2" s="8">
-        <v>5.33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="C3" s="71">
+        <v>9.57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="25" t="s">
+        <v>322</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="29" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="C3" s="6">
-        <v>5.35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>328</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>230</v>
-      </c>
-      <c r="C5" s="31" t="str">
+      <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
         <v/>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="37" t="s">
-        <v>231</v>
-      </c>
-      <c r="C6" s="38" t="str">
+      <c r="B6" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
         <v>Baja</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="C7" s="72">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C8" s="71">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>233</v>
+      </c>
+      <c r="C10" s="30">
+        <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="36" t="s">
         <v>234</v>
       </c>
-      <c r="C7" s="8">
-        <v>0.86</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
-        <v>233</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="C11" s="37" t="str">
+        <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
+        <v>Permanece</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="25" t="s">
         <v>235</v>
       </c>
-      <c r="C8" s="6">
-        <v>0.79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="26" t="s">
-        <v>317</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="30" t="s">
+      <c r="B12" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="25" t="s">
         <v>236</v>
       </c>
-      <c r="C10" s="31">
-        <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="37" t="s">
+      <c r="B13" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="C11" s="38" t="str">
-        <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Sube</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="C12" s="8">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="C13" s="6">
-        <v>0.2</v>
+      <c r="C13" s="6" t="s">
+        <v>435</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="C14" s="9"/>
+    </row>
+    <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="27" t="s">
+        <v>244</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C15" s="10"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="26" t="s">
+        <v>241</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="27" t="s">
+        <v>242</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="C14" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="26" t="s">
-        <v>241</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
-        <v>242</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="27" t="s">
-        <v>249</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>251</v>
-      </c>
       <c r="C17" s="10"/>
     </row>
-    <row r="18" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="28" t="s">
-        <v>250</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="C18" s="11"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="27" t="s">
+    <row r="18" spans="1:3" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="28" t="s">
+      <c r="C18" s="70" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="C20" s="11"/>
-    </row>
-    <row r="21" spans="1:3" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="C21" s="71" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>254</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>371</v>
+      <c r="C19" s="13" t="s">
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -4702,13 +4617,13 @@
           <x14:formula1>
             <xm:f>Tablas!$A$2:$A$7</xm:f>
           </x14:formula1>
-          <xm:sqref>C22</xm:sqref>
+          <xm:sqref>C19</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{84A5E201-9A26-4AA5-938D-DF5311A91175}">
           <x14:formula1>
             <xm:f>Tablas!$L$30</xm:f>
           </x14:formula1>
-          <xm:sqref>C21</xm:sqref>
+          <xm:sqref>C18</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4722,7 +4637,7 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="56.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" style="15" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" style="14" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" style="5" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="5"/>
   </cols>
@@ -4739,168 +4654,168 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
+        <v>366</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="C2" s="72">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
+        <v>367</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C3" s="71">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="25" t="s">
+        <v>368</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>374</v>
+      </c>
+      <c r="C5" s="30" t="str">
+        <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>375</v>
+      </c>
+      <c r="C6" s="37" t="str">
+        <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
+        <v>Baja</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="C7" s="74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="C2" s="73">
-        <v>-0.08</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
-        <v>373</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="C8" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="C3" s="72">
-        <v>-0.08</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>374</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="C9" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="30" t="s">
+      <c r="C10" s="75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>380</v>
       </c>
-      <c r="C5" s="31">
-        <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
+      <c r="C11" s="75">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="37" t="s">
+    <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="C6" s="38" t="str">
-        <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Permanece</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="C12" s="76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="26" t="s">
+        <v>369</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="27" t="s">
+        <v>370</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>382</v>
       </c>
-      <c r="C7" s="75">
-        <v>9.8000000000000007</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>383</v>
-      </c>
-      <c r="C8" s="76">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="C14" s="10"/>
+    </row>
+    <row r="15" spans="1:3" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>384</v>
       </c>
-      <c r="C9" s="76">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="B10" s="5" t="s">
+      <c r="C15" s="11" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>385</v>
       </c>
-      <c r="C10" s="76">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>386</v>
-      </c>
-      <c r="C11" s="76">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>387</v>
-      </c>
-      <c r="C12" s="77">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
-        <v>375</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>389</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
-        <v>376</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>388</v>
-      </c>
-      <c r="C14" s="11"/>
-    </row>
-    <row r="15" spans="1:3" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>390</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>391</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>371</v>
+      <c r="C16" s="13" t="s">
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -4932,507 +4847,507 @@
   <dimension ref="A1:M30"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="140.85546875" style="46" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11.42578125" style="46"/>
-    <col min="4" max="4" width="14.85546875" style="46" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" style="46" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="91.5703125" style="46" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" style="46" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" style="46" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="46.42578125" style="46" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="48.85546875" style="46" customWidth="1"/>
-    <col min="11" max="11" width="45.85546875" style="46" customWidth="1"/>
-    <col min="12" max="12" width="103.7109375" style="54" customWidth="1"/>
-    <col min="13" max="16384" width="11.42578125" style="46"/>
+    <col min="1" max="1" width="140.85546875" style="45" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.42578125" style="45"/>
+    <col min="4" max="4" width="14.85546875" style="45" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" style="45" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="91.5703125" style="45" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" style="45" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="20.85546875" style="45" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="46.42578125" style="45" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="48.85546875" style="45" customWidth="1"/>
+    <col min="11" max="11" width="45.85546875" style="45" customWidth="1"/>
+    <col min="12" max="12" width="103.7109375" style="53" customWidth="1"/>
+    <col min="13" max="16384" width="11.42578125" style="45"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="44" t="s">
+        <v>250</v>
+      </c>
+      <c r="C1" s="44" t="s">
+        <v>283</v>
+      </c>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
+      <c r="J1" s="49"/>
+      <c r="K1" s="49"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="49"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="45" t="s">
+        <v>251</v>
+      </c>
+      <c r="C2" s="47" t="s">
+        <v>268</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>265</v>
+      </c>
+      <c r="E2" s="47" t="s">
+        <v>266</v>
+      </c>
+      <c r="F2" s="48" t="s">
+        <v>255</v>
+      </c>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="45" t="s">
+        <v>365</v>
+      </c>
+      <c r="C3" s="45" t="s">
+        <v>267</v>
+      </c>
+      <c r="D3" s="45">
+        <v>70</v>
+      </c>
+      <c r="E3" s="45">
+        <v>200</v>
+      </c>
+      <c r="F3" s="45" t="s">
+        <v>277</v>
+      </c>
+      <c r="I3" s="45" t="s">
+        <v>302</v>
+      </c>
+      <c r="J3" s="45" t="s">
+        <v>259</v>
+      </c>
+      <c r="K3" s="45" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="45" t="s">
+        <v>252</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>267</v>
+      </c>
+      <c r="D4" s="45">
+        <v>30</v>
+      </c>
+      <c r="E4" s="45">
+        <v>100</v>
+      </c>
+      <c r="F4" s="45" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="45" t="s">
+        <v>253</v>
+      </c>
+      <c r="F5" s="45" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="45" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" s="45" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="47" t="s">
+        <v>269</v>
+      </c>
+      <c r="F7" s="46" t="s">
         <v>256</v>
       </c>
-      <c r="C1" s="45" t="s">
-        <v>289</v>
-      </c>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="50"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="46" t="s">
+      <c r="G7" s="46"/>
+      <c r="H7" s="46"/>
+      <c r="I7" s="46"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="46"/>
+      <c r="L7" s="68"/>
+      <c r="M7" s="46"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E8" s="45" t="s">
+        <v>304</v>
+      </c>
+      <c r="F8" s="45" t="s">
+        <v>303</v>
+      </c>
+      <c r="I8" s="45" t="s">
+        <v>307</v>
+      </c>
+      <c r="J8" s="45" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E9" s="45" t="s">
+        <v>305</v>
+      </c>
+      <c r="I9" s="45" t="s">
+        <v>308</v>
+      </c>
+      <c r="J9" s="45" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E10" s="45" t="s">
+        <v>306</v>
+      </c>
+      <c r="I10" s="45" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="C12" s="47" t="s">
+        <v>270</v>
+      </c>
+      <c r="D12" s="47" t="s">
+        <v>268</v>
+      </c>
+      <c r="E12" s="47" t="s">
+        <v>271</v>
+      </c>
+      <c r="F12" s="46" t="s">
         <v>257</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="G12" s="46"/>
+      <c r="H12" s="46"/>
+      <c r="I12" s="46"/>
+      <c r="J12" s="46"/>
+      <c r="K12" s="46"/>
+      <c r="L12" s="68"/>
+      <c r="M12" s="46"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="D13" s="45" t="s">
+        <v>267</v>
+      </c>
+      <c r="F13" s="45" t="s">
+        <v>356</v>
+      </c>
+      <c r="I13" s="45" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="D14" s="45" t="s">
+        <v>272</v>
+      </c>
+      <c r="I14" s="45" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="D15" s="45" t="s">
+        <v>273</v>
+      </c>
+      <c r="I15" s="45" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="17" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C17" s="47" t="s">
+        <v>270</v>
+      </c>
+      <c r="D17" s="47" t="s">
+        <v>268</v>
+      </c>
+      <c r="E17" s="47" t="s">
+        <v>271</v>
+      </c>
+      <c r="F17" s="46" t="s">
+        <v>258</v>
+      </c>
+      <c r="G17" s="46"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="46"/>
+      <c r="K17" s="46"/>
+      <c r="L17" s="68"/>
+      <c r="M17" s="46"/>
+    </row>
+    <row r="18" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F18" s="45" t="s">
+        <v>261</v>
+      </c>
+      <c r="I18" s="45" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="19" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F19" s="45" t="s">
+        <v>263</v>
+      </c>
+      <c r="I19" s="45" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="22" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C22" s="50" t="s">
+        <v>284</v>
+      </c>
+      <c r="D22" s="50" t="s">
+        <v>275</v>
+      </c>
+      <c r="E22" s="50" t="s">
         <v>274</v>
       </c>
-      <c r="D2" s="48" t="s">
-        <v>271</v>
-      </c>
-      <c r="E2" s="48" t="s">
-        <v>272</v>
-      </c>
-      <c r="F2" s="49" t="s">
-        <v>261</v>
-      </c>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="46" t="s">
-        <v>371</v>
-      </c>
-      <c r="C3" s="46" t="s">
-        <v>273</v>
-      </c>
-      <c r="D3" s="46">
-        <v>70</v>
-      </c>
-      <c r="E3" s="46">
-        <v>200</v>
-      </c>
-      <c r="F3" s="46" t="s">
-        <v>283</v>
-      </c>
-      <c r="I3" s="46" t="s">
-        <v>308</v>
-      </c>
-      <c r="J3" s="46" t="s">
-        <v>265</v>
-      </c>
-      <c r="K3" s="46" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="46" t="s">
-        <v>258</v>
-      </c>
-      <c r="C4" s="46" t="s">
-        <v>273</v>
-      </c>
-      <c r="D4" s="46">
-        <v>30</v>
-      </c>
-      <c r="E4" s="46">
-        <v>100</v>
-      </c>
-      <c r="F4" s="46" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="46" t="s">
-        <v>259</v>
-      </c>
-      <c r="F5" s="46" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="46" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="46" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="48" t="s">
-        <v>275</v>
-      </c>
-      <c r="F7" s="47" t="s">
-        <v>262</v>
-      </c>
-      <c r="G7" s="47"/>
-      <c r="H7" s="47"/>
-      <c r="I7" s="47"/>
-      <c r="J7" s="47"/>
-      <c r="K7" s="47"/>
-      <c r="L7" s="69"/>
-      <c r="M7" s="47"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E8" s="46" t="s">
-        <v>310</v>
-      </c>
-      <c r="F8" s="46" t="s">
-        <v>309</v>
-      </c>
-      <c r="I8" s="46" t="s">
-        <v>313</v>
-      </c>
-      <c r="J8" s="46" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E9" s="46" t="s">
-        <v>311</v>
-      </c>
-      <c r="I9" s="46" t="s">
-        <v>314</v>
-      </c>
-      <c r="J9" s="46" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E10" s="46" t="s">
-        <v>312</v>
-      </c>
-      <c r="I10" s="46" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C12" s="48" t="s">
-        <v>276</v>
-      </c>
-      <c r="D12" s="48" t="s">
-        <v>274</v>
-      </c>
-      <c r="E12" s="48" t="s">
-        <v>277</v>
-      </c>
-      <c r="F12" s="47" t="s">
-        <v>263</v>
-      </c>
-      <c r="G12" s="47"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="47"/>
-      <c r="J12" s="47"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="69"/>
-      <c r="M12" s="47"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D13" s="46" t="s">
-        <v>273</v>
-      </c>
-      <c r="F13" s="46" t="s">
-        <v>362</v>
-      </c>
-      <c r="I13" s="46" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D14" s="46" t="s">
-        <v>278</v>
-      </c>
-      <c r="I14" s="46" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D15" s="46" t="s">
-        <v>279</v>
-      </c>
-      <c r="I15" s="46" t="s">
+      <c r="F22" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="G22" s="50"/>
+      <c r="H22" s="50"/>
+      <c r="I22" s="50" t="s">
+        <v>299</v>
+      </c>
+      <c r="J22" s="50" t="s">
+        <v>300</v>
+      </c>
+      <c r="K22" s="50" t="s">
+        <v>301</v>
+      </c>
+      <c r="L22" s="69" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="17" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C17" s="48" t="s">
-        <v>276</v>
-      </c>
-      <c r="D17" s="48" t="s">
-        <v>274</v>
-      </c>
-      <c r="E17" s="48" t="s">
-        <v>277</v>
-      </c>
-      <c r="F17" s="47" t="s">
-        <v>264</v>
-      </c>
-      <c r="G17" s="47"/>
-      <c r="H17" s="47"/>
-      <c r="I17" s="47"/>
-      <c r="J17" s="47"/>
-      <c r="K17" s="47"/>
-      <c r="L17" s="69"/>
-      <c r="M17" s="47"/>
-    </row>
-    <row r="18" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="F18" s="46" t="s">
-        <v>267</v>
-      </c>
-      <c r="I18" s="46" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="19" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="F19" s="46" t="s">
-        <v>269</v>
-      </c>
-      <c r="I19" s="46" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="22" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C22" s="51" t="s">
-        <v>290</v>
-      </c>
-      <c r="D22" s="51" t="s">
-        <v>281</v>
-      </c>
-      <c r="E22" s="51" t="s">
-        <v>280</v>
-      </c>
-      <c r="F22" s="51" t="s">
-        <v>304</v>
-      </c>
-      <c r="G22" s="51"/>
-      <c r="H22" s="51"/>
-      <c r="I22" s="51" t="s">
-        <v>305</v>
-      </c>
-      <c r="J22" s="51" t="s">
-        <v>306</v>
-      </c>
-      <c r="K22" s="51" t="s">
-        <v>307</v>
-      </c>
-      <c r="L22" s="70" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="23" spans="3:13" s="64" customFormat="1" ht="99" x14ac:dyDescent="0.25">
-      <c r="C23" s="64" t="s">
-        <v>293</v>
-      </c>
-      <c r="D23" s="64" t="s">
-        <v>292</v>
-      </c>
-      <c r="E23" s="64" t="s">
-        <v>288</v>
-      </c>
-      <c r="F23" s="53" t="str">
+    <row r="23" spans="3:13" s="63" customFormat="1" ht="99" x14ac:dyDescent="0.25">
+      <c r="C23" s="63" t="s">
+        <v>287</v>
+      </c>
+      <c r="D23" s="63" t="s">
+        <v>286</v>
+      </c>
+      <c r="E23" s="63" t="s">
+        <v>282</v>
+      </c>
+      <c r="F23" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 34.7 mm y con un máximo de 19 mm/día.</v>
-      </c>
-      <c r="G23" s="53"/>
-      <c r="H23" s="53"/>
-      <c r="I23" s="53" t="str">
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día.</v>
+      </c>
+      <c r="G23" s="52"/>
+      <c r="H23" s="52"/>
+      <c r="I23" s="52" t="str">
         <f>_xlfn.CONCAT($F$8,D23,IF(YI!C15=$E$8,$I$8,IF(YI!C15=$E$9,$I$9,$I$10)),$J$8,E23,". ")</f>
         <v xml:space="preserve">Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno. </v>
       </c>
-      <c r="J23" s="53" t="str">
+      <c r="J23" s="52" t="str">
         <f>_xlfn.CONCAT(F13,IF(YI!C31&gt;YI!C11,I13, IF(YI!C31=YI!C11,I14, I15)))</f>
         <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días. </v>
       </c>
-      <c r="K23" s="53" t="str">
+      <c r="K23" s="52" t="str">
         <f>IF(YI!C13="-","",IF(YI!C31&gt;YI!C13,_xlfn.CONCAT(F18,YI!C13,I18),_xlfn.CONCAT(F19,YI!C13,I19)))</f>
         <v xml:space="preserve">Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
-      <c r="L23" s="53" t="str">
+      <c r="L23" s="52" t="str">
         <f>+_xlfn.CONCAT(F23," ",I23, " ",J23," ",K23)</f>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 34.7 mm y con un máximo de 19 mm/día. Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Yí, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Yí se mantiene constante en la ciudad de Durazno.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="C24" s="52" t="s">
-        <v>294</v>
-      </c>
-      <c r="D24" s="52" t="s">
-        <v>295</v>
-      </c>
-      <c r="E24" s="52" t="s">
-        <v>287</v>
-      </c>
-      <c r="F24" s="54" t="str">
+      <c r="C24" s="51" t="s">
+        <v>288</v>
+      </c>
+      <c r="D24" s="51" t="s">
+        <v>289</v>
+      </c>
+      <c r="E24" s="51" t="s">
+        <v>281</v>
+      </c>
+      <c r="F24" s="53" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 88 mm y con un máximo de 65 mm/día.</v>
-      </c>
-      <c r="G24" s="54"/>
-      <c r="H24" s="54"/>
-      <c r="I24" s="65" t="str">
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día.</v>
+      </c>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D24,IF(CUAREIM!C16=$E$8,$I$8,IF(CUAREIM!C16=$E$9,$I$9,$I$10)),$J$8,E24,". ")</f>
         <v xml:space="preserve">Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas. </v>
       </c>
-      <c r="J24" s="54" t="str">
+      <c r="J24" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(CUAREIM!C27&gt;CUAREIM!C12,I13, IF(CUAREIM!C27=CUAREIM!C12,I14, I15)))</f>
         <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días. </v>
       </c>
-      <c r="K24" s="53" t="str">
+      <c r="K24" s="52" t="str">
         <f>IF(CUAREIM!C14="-","",IF(CUAREIM!C27&gt;CUAREIM!C14,_xlfn.CONCAT(F18,CUAREIM!C14,I18),_xlfn.CONCAT(F19,CUAREIM!C14,I19)))</f>
         <v/>
       </c>
-      <c r="L24" s="53" t="str">
+      <c r="L24" s="52" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 88 mm y con un máximo de 65 mm/día. Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">
-      <c r="C25" s="52" t="s">
-        <v>286</v>
-      </c>
-      <c r="D25" s="52" t="s">
-        <v>296</v>
-      </c>
-      <c r="E25" s="52" t="s">
-        <v>286</v>
-      </c>
-      <c r="F25" s="53" t="str">
+      <c r="C25" s="51" t="s">
+        <v>280</v>
+      </c>
+      <c r="D25" s="51" t="s">
+        <v>290</v>
+      </c>
+      <c r="E25" s="51" t="s">
+        <v>280</v>
+      </c>
+      <c r="F25" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$3,SUM(SANTALUCIA!C22:C24)&gt;$E$3),$F$3,IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$4,SUM(SANTALUCIA!C22:C24)&gt;$E$4),$F$4,$F$5)),D25,$I$3,SUM(SANTALUCIA!C22:C24),$J$3,MAX(SANTALUCIA!C22:C24),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 9.8 mm y con un máximo de 9.8 mm/día.</v>
-      </c>
-      <c r="G25" s="53"/>
-      <c r="H25" s="53"/>
-      <c r="I25" s="65" t="str">
+        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día.</v>
+      </c>
+      <c r="G25" s="52"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D25,IF(SANTALUCIA!C16=$E$8,$I$8,IF(SANTALUCIA!C16=$E$9,$I$9,$I$10)),$J$8,E25,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía. </v>
-      </c>
-      <c r="J25" s="54" t="str">
+        <v xml:space="preserve">Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía. </v>
+      </c>
+      <c r="J25" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(SANTALUCIA!C36&gt;SANTALUCIA!C12,I13, IF(SANTALUCIA!C36=SANTALUCIA!C12,I14, I15)))</f>
         <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días. </v>
       </c>
-      <c r="K25" s="54" t="str">
+      <c r="K25" s="53" t="str">
         <f>IF(SANTALUCIA!C14="-","",IF(SANTALUCIA!C36&gt;SANTALUCIA!C14,_xlfn.CONCAT(F18,SANTALUCIA!C14,I18),_xlfn.CONCAT(F19,SANTALUCIA!C14,I19)))</f>
         <v xml:space="preserve">Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
-      <c r="L25" s="53" t="str">
+      <c r="L25" s="52" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 9.8 mm y con un máximo de 9.8 mm/día. Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="26" spans="3:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C26" s="52" t="s">
-        <v>297</v>
-      </c>
-      <c r="D26" s="52" t="s">
-        <v>298</v>
-      </c>
-      <c r="E26" s="52" t="s">
-        <v>299</v>
-      </c>
-      <c r="F26" s="78" t="str">
-        <f>_xlfn.CONCAT(IF(OR(MAX(URUGUAY!C27:C29)&gt;$D$3,SUM(URUGUAY!C27:C29)&gt;$E$3),$F$3,IF(OR(MAX(URUGUAY!C27:C29)&gt;$D$4,SUM(URUGUAY!C27:C29)&gt;$E$4),$F$4,$F$5)),D26,$I$3,SUM(URUGUAY!C27:C29),$J$3,MAX(URUGUAY!C27:C29),$K$3)</f>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Uruguay, donde en las últimas 72 horas se acumularon 36.4 mm y con un máximo de 31.3 mm/día.</v>
-      </c>
-      <c r="I26" s="65" t="str">
+      <c r="C26" s="51" t="s">
+        <v>291</v>
+      </c>
+      <c r="D26" s="51" t="s">
+        <v>292</v>
+      </c>
+      <c r="E26" s="51" t="s">
+        <v>293</v>
+      </c>
+      <c r="F26" s="77" t="e">
+        <f>_xlfn.CONCAT(IF(OR(MAX(URUGUAY!#REF!)&gt;$D$3,SUM(URUGUAY!#REF!)&gt;$E$3),$F$3,IF(OR(MAX(URUGUAY!#REF!)&gt;$D$4,SUM(URUGUAY!#REF!)&gt;$E$4),$F$4,$F$5)),D26,$I$3,SUM(URUGUAY!#REF!),$J$3,MAX(URUGUAY!#REF!),$K$3)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="I26" s="64" t="str">
         <f>IF(AND(URUGUAY!$C$11=$E$8,URUGUAY!$C$16=$E$8,URUGUAY!$C$21=$E$8,URUGUAY!$C$26=$E$8),_xlfn.CONCAT($F$8,$D$26,$I$8,$J$9," ",E26,", ",E27,", ",E28," y ",Tablas!E29,"."),IF(AND(URUGUAY!$C$11=$E$9,URUGUAY!$C$16=$E$9,URUGUAY!$C$21=$E$9,URUGUAY!$C$26=$E$9),_xlfn.CONCAT($F$8,$D$26,$I$9,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),IF(AND(URUGUAY!$C$11=$E$10,URUGUAY!$C$16=$E$10,URUGUAY!$C$21=$E$10,URUGUAY!$C$26=$E$10),_xlfn.CONCAT($F$8,$D$26,$I$10,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),_xlfn.CONCAT($F$8,D26,I27,I28,I29))))</f>
-        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Salto Paysandú; se mantiene constante en la ciudad de ; está en descenso en la ciudad de  Fray Bentos.</v>
-      </c>
-      <c r="J26" s="79" t="str">
-        <f>_xlfn.CONCAT(F13,IF(AND(URUGUAY!C31&gt;URUGUAY!C7, URUGUAY!C33&gt;URUGUAY!C12, URUGUAY!C35&gt;URUGUAY!C17, URUGUAY!C37&gt;URUGUAY!C22),I13, IF(AND(URUGUAY!C31=URUGUAY!C7, URUGUAY!C33=URUGUAY!C12, URUGUAY!C35=URUGUAY!C17, URUGUAY!C37=URUGUAY!C22),I14, I15)))</f>
+        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Salto Paysandú; se mantiene constante en la ciudad de  Bella Unión; está en descenso en la ciudad de  Fray Bentos.</v>
+      </c>
+      <c r="J26" s="78" t="str">
+        <f>_xlfn.CONCAT(F13,IF(AND(URUGUAY!C28&gt;URUGUAY!C7, URUGUAY!C30&gt;URUGUAY!C12, URUGUAY!C32&gt;URUGUAY!C17, URUGUAY!C34&gt;URUGUAY!C22),I13, IF(AND(URUGUAY!C28=URUGUAY!C7, URUGUAY!C30=URUGUAY!C12, URUGUAY!C32=URUGUAY!C17, URUGUAY!C34=URUGUAY!C22),I14, I15)))</f>
         <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, se prevé que el nivel descienda en los próximos días. </v>
       </c>
-      <c r="K26" s="79" t="str">
-        <f>IF(AND(URUGUAY!C9="-", URUGUAY!C14="-", URUGUAY!C19="-", URUGUAY!C24="-"),"",IF(OR(URUGUAY!C31&gt;URUGUAY!C9, URUGUAY!C33&gt;URUGUAY!C14, URUGUAY!C35&gt;URUGUAY!C19,URUGUAY!C37&gt;URUGUAY!C24),_xlfn.CONCAT(F18,IF(URUGUAY!C9&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C9,"m en ",E26," "),""), IF(URUGUAY!C14&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C14, "m en ",E27," "),""),IF(URUGUAY!C19&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C19,"m en ",E28," "),""),IF(URUGUAY!C24&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C24,"m en ",E29),""),")."),_xlfn.CONCAT(F19,IF(URUGUAY!C9&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C9,"m en ",E26," "),""), IF(URUGUAY!C14&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C14, "m en ",E27," "),""),IF(URUGUAY!C19&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C19,"m en ",E28," "),""),IF(URUGUAY!C24&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C24,"m en ",E29),""),", pero no se puede descartar en su totalidad.")))</f>
+      <c r="K26" s="78" t="str">
+        <f>IF(AND(URUGUAY!C9="-", URUGUAY!C14="-", URUGUAY!C19="-", URUGUAY!C24="-"),"",IF(OR(URUGUAY!C28&gt;URUGUAY!C9, URUGUAY!C30&gt;URUGUAY!C14, URUGUAY!C32&gt;URUGUAY!C19,URUGUAY!C34&gt;URUGUAY!C24),_xlfn.CONCAT(F18,IF(URUGUAY!C9&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C9,"m en ",E26," "),""), IF(URUGUAY!C14&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C14, "m en ",E27," "),""),IF(URUGUAY!C19&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C19,"m en ",E28," "),""),IF(URUGUAY!C24&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C24,"m en ",E29),""),")."),_xlfn.CONCAT(F19,IF(URUGUAY!C9&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C9,"m en ",E26," "),""), IF(URUGUAY!C14&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C14, "m en ",E27," "),""),IF(URUGUAY!C19&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C19,"m en ",E28," "),""),IF(URUGUAY!C24&lt;&gt;"-",_xlfn.CONCAT(URUGUAY!C24,"m en ",E29),""),", pero no se puede descartar en su totalidad.")))</f>
         <v>Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( -m en Paysandú ).</v>
       </c>
-      <c r="L26" s="79" t="str">
+      <c r="L26" s="78" t="e">
         <f t="shared" si="0"/>
-        <v>En las últimas horas se registraron acumulados de precipitación moderados en la cuenca del río Uruguay, donde en las últimas 72 horas se acumularon 36.4 mm y con un máximo de 31.3 mm/día. Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Bella Unión Salto Paysandú; se mantiene constante en la ciudad de ; está en descenso en la ciudad de  Fray Bentos. Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, se prevé que el nivel descienda en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( -m en Paysandú ).</v>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="27" spans="3:13" ht="33" x14ac:dyDescent="0.3">
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="52" t="s">
-        <v>300</v>
-      </c>
-      <c r="F27" s="78"/>
-      <c r="G27" s="59">
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51" t="s">
+        <v>294</v>
+      </c>
+      <c r="F27" s="77"/>
+      <c r="G27" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E8, URUGUAY!$C$16=Tablas!E8,URUGUAY!$C$21=Tablas!E8,URUGUAY!$C$26=Tablas!E8)</f>
-        <v>3</v>
-      </c>
-      <c r="H27" s="60" t="str">
+        <v>2</v>
+      </c>
+      <c r="H27" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E8,_xlfn.CONCAT(" ",$E$26,),""),IF(URUGUAY!$C$16=Tablas!E8,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E8,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E8,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Bella Unión Salto Paysandú</v>
-      </c>
-      <c r="I27" s="66" t="str">
+        <v xml:space="preserve"> Salto Paysandú</v>
+      </c>
+      <c r="I27" s="65" t="str">
         <f>_xlfn.CONCAT(I8,IF(G27&gt;1,$J$9,$J$8),H27, IF(G27=4,".", ";"))</f>
-        <v xml:space="preserve"> está en ascenso en las ciudades de Bella Unión Salto Paysandú;</v>
-      </c>
-      <c r="J27" s="79"/>
-      <c r="K27" s="79"/>
-      <c r="L27" s="79"/>
-    </row>
-    <row r="28" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
-      <c r="E28" s="52" t="s">
-        <v>301</v>
-      </c>
-      <c r="F28" s="78"/>
-      <c r="G28" s="59">
+        <v xml:space="preserve"> está en ascenso en las ciudades de Salto Paysandú;</v>
+      </c>
+      <c r="J27" s="78"/>
+      <c r="K27" s="78"/>
+      <c r="L27" s="78"/>
+    </row>
+    <row r="28" spans="3:13" ht="33" x14ac:dyDescent="0.3">
+      <c r="C28" s="51"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="51" t="s">
+        <v>295</v>
+      </c>
+      <c r="F28" s="77"/>
+      <c r="G28" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E9, URUGUAY!$C$16=Tablas!E9,URUGUAY!$C$21=Tablas!E9,URUGUAY!$C$26=Tablas!E9)</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="60" t="str">
+        <v>1</v>
+      </c>
+      <c r="H28" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E9,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E9,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E9,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E9,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v/>
-      </c>
-      <c r="I28" s="66" t="str">
+        <v xml:space="preserve"> Bella Unión</v>
+      </c>
+      <c r="I28" s="65" t="str">
         <f>_xlfn.CONCAT(I9,IF(G28&gt;1,$J$9,$J$8),H28, IF((G27+G28)=4,".", ";"))</f>
-        <v xml:space="preserve"> se mantiene constante en la ciudad de ;</v>
-      </c>
-      <c r="J28" s="79"/>
-      <c r="K28" s="79"/>
-      <c r="L28" s="79"/>
+        <v xml:space="preserve"> se mantiene constante en la ciudad de  Bella Unión;</v>
+      </c>
+      <c r="J28" s="78"/>
+      <c r="K28" s="78"/>
+      <c r="L28" s="78"/>
     </row>
     <row r="29" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="52" t="s">
-        <v>302</v>
-      </c>
-      <c r="F29" s="78"/>
-      <c r="G29" s="59">
+      <c r="C29" s="51"/>
+      <c r="D29" s="51"/>
+      <c r="E29" s="51" t="s">
+        <v>296</v>
+      </c>
+      <c r="F29" s="77"/>
+      <c r="G29" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E10, URUGUAY!$C$16=Tablas!E10,URUGUAY!$C$21=Tablas!E10,URUGUAY!$C$26=Tablas!E10)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="60" t="str">
+      <c r="H29" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E10,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E10,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E10,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E10,_xlfn.CONCAT(" ",$E$29),""))</f>
         <v xml:space="preserve"> Fray Bentos</v>
       </c>
-      <c r="I29" s="66" t="str">
+      <c r="I29" s="65" t="str">
         <f>_xlfn.CONCAT(I10,IF(G29&gt;1,$J$9,$J$8),H29, ".")</f>
         <v xml:space="preserve"> está en descenso en la ciudad de  Fray Bentos.</v>
       </c>
-      <c r="J29" s="79"/>
-      <c r="K29" s="79"/>
-      <c r="L29" s="79"/>
+      <c r="J29" s="78"/>
+      <c r="K29" s="78"/>
+      <c r="L29" s="78"/>
     </row>
     <row r="30" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="C30" s="52" t="s">
-        <v>303</v>
-      </c>
-      <c r="D30" s="52" t="s">
-        <v>303</v>
-      </c>
-      <c r="E30" s="52" t="s">
-        <v>282</v>
-      </c>
-      <c r="F30" s="53" t="str">
-        <f>_xlfn.CONCAT(IF(OR(MAX(NEGRO!C12:C14)&gt;$D$3,SUM(NEGRO!C12:C14)&gt;$E$3),$F$3,IF(OR(MAX(NEGRO!C12:C14)&gt;$D$4,SUM(NEGRO!C12:C14)&gt;$E$4),$F$4,$F$5)),D30,$I$3,SUM(NEGRO!C12:C14),$J$3,MAX(NEGRO!C12:C14),$K$3)</f>
-        <v>En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del Río Negro, donde en las últimas 72 horas se acumularon 1.6 mm y con un máximo de 1.4 mm/día.</v>
-      </c>
-      <c r="G30" s="53"/>
-      <c r="H30" s="53"/>
-      <c r="I30" s="65" t="str">
+      <c r="C30" s="51" t="s">
+        <v>297</v>
+      </c>
+      <c r="D30" s="51" t="s">
+        <v>297</v>
+      </c>
+      <c r="E30" s="51" t="s">
+        <v>276</v>
+      </c>
+      <c r="F30" s="52" t="e">
+        <f>_xlfn.CONCAT(IF(OR(MAX(NEGRO!#REF!)&gt;$D$3,SUM(NEGRO!#REF!)&gt;$E$3),$F$3,IF(OR(MAX(NEGRO!#REF!)&gt;$D$4,SUM(NEGRO!#REF!)&gt;$E$4),$F$4,$F$5)),D30,$I$3,SUM(NEGRO!#REF!),$J$3,MAX(NEGRO!#REF!),$K$3)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="G30" s="52"/>
+      <c r="H30" s="52"/>
+      <c r="I30" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D30,IF(NEGRO!C11=$E$8,$I$8,IF(NEGRO!C11=$E$9,$I$9,$I$10)),$J$8,E30,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del Río Negro está en ascenso en la ciudad de Mercedes. </v>
-      </c>
-      <c r="J30" s="54" t="str">
-        <f>_xlfn.CONCAT(F13,IF(NEGRO!C19&gt;NEGRO!C7,I13, IF(NEGRO!C19=NEGRO!C7,I14, I15)))</f>
+        <v xml:space="preserve">Actualmente, el nivel del Río Negro se mantiene constante en la ciudad de Mercedes. </v>
+      </c>
+      <c r="J30" s="53" t="str">
+        <f>_xlfn.CONCAT(F13,IF(NEGRO!C16&gt;NEGRO!C7,I13, IF(NEGRO!C16=NEGRO!C7,I14, I15)))</f>
         <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días. </v>
       </c>
-      <c r="K30" s="67" t="str">
-        <f>IF(NEGRO!C9="-","",IF(NEGRO!C19&gt;NEGRO!C9,_xlfn.CONCAT(F18,NEGRO!C9,I18),_xlfn.CONCAT(F19,NEGRO!C9,I19)))</f>
+      <c r="K30" s="66" t="str">
+        <f>IF(NEGRO!C9="-","",IF(NEGRO!C16&gt;NEGRO!C9,_xlfn.CONCAT(F18,NEGRO!C9,I18),_xlfn.CONCAT(F19,NEGRO!C9,I19)))</f>
         <v/>
       </c>
-      <c r="L30" s="53" t="str">
+      <c r="L30" s="52" t="e">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del Río Negro, donde en las últimas 72 horas se acumularon 1.6 mm y con un máximo de 1.4 mm/día. Actualmente, el nivel del Río Negro está en ascenso en la ciudad de Mercedes.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v>#REF!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update codes for importing data from fews2floodreport
</commit_message>
<xml_diff>
--- a/automatic docx/database_report.xlsx
+++ b/automatic docx/database_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Sala_Situacion_Dinagua\automatic docx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E523873F-69BF-4E33-AD00-BCA55854B3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7188EF8B-540B-46DA-B0AA-885C6ACB39F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{83108E16-E9D6-4CCB-B5BE-A67101359CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="INICIO" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="434">
   <si>
     <t>fecha_emision</t>
   </si>
@@ -165,9 +165,6 @@
     <t>diagnostico_yi</t>
   </si>
   <si>
-    <t xml:space="preserve">Estar preparados ante la posibilidad de otro incremento que pueda experimentar el río debido a las lluvias registradas en las ultimas horas.  </t>
-  </si>
-  <si>
     <t>recomendacion_yi</t>
   </si>
   <si>
@@ -801,15 +798,6 @@
     <t xml:space="preserve">Estar atentos a los próximos eventos de lluvia que se registren en la cuenca.   </t>
   </si>
   <si>
-    <t xml:space="preserve">Mantener el monitoreo hidrológico reforzado en la zona y estar atento a las actualizaciones de pronósticos del tiempo para los próximos días. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estar atentos a posibles inundaciones locales en </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estar atentos a la posibilidad de un nuevo incremento de nivel del río Yí el cual podría generar impactos en la zona de camping de la ciudad. </t>
-  </si>
-  <si>
     <t xml:space="preserve">En las últimas horas se registraron precipitaciones de fuerte intensidad en la cuenca (promedio 62 mm) del río Cuareim. </t>
   </si>
   <si>
@@ -1254,9 +1242,6 @@
     <t xml:space="preserve"> -</t>
   </si>
   <si>
-    <t>Menor a 3.5 m</t>
-  </si>
-  <si>
     <t>29/05</t>
   </si>
   <si>
@@ -1302,9 +1287,6 @@
     <t>Entre 5.50 y 6.10 metros</t>
   </si>
   <si>
-    <t>Entre 8.50 y 9.70 metros</t>
-  </si>
-  <si>
     <t>Entre 4.50 y 5.00 metros</t>
   </si>
   <si>
@@ -1344,13 +1326,25 @@
     <t xml:space="preserve">Durante las últimas horas se registró el nivel máximo del río Cuareim en Artigas el cual alcanzó los 6.14 metros, sin acercarse a la cota de aviso (8.00 m). Actualmente el nivel del río se encuentra en descenso y no se espera nuevo incrementos en los próximos días. </t>
   </si>
   <si>
-    <t>2000 y 3000</t>
-  </si>
-  <si>
-    <t>1000 y 2000</t>
-  </si>
-  <si>
-    <t>500 y 1000</t>
+    <t>24000 y 30000</t>
+  </si>
+  <si>
+    <t>150 y 375</t>
+  </si>
+  <si>
+    <t>375 y 500</t>
+  </si>
+  <si>
+    <t>Mantener la vigilancia y el monitoreo en niveles de ríos y arroyos. Infórmese por fuentes oficiales</t>
+  </si>
+  <si>
+    <t>Estar atentos a la posiblidad de generarse inundaciones en los primeros equipamientos colectivos expuesto de la localidad y pérdida de conectividad terrestre por crecidas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estar preparados ante la posibilidad de generarse inundaciones en zona de vivienda de uso permanente ubicada en la trama urbana. </t>
+  </si>
+  <si>
+    <t>Tomar acción en realizar evacuaciones debido a la posibilidad de generarse inundaciones que afecten viviendas, infraestructura sensible y equipamientos urbanos</t>
   </si>
 </sst>
 </file>
@@ -2197,7 +2191,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>9</v>
@@ -2208,7 +2202,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="34" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>8</v>
@@ -2219,7 +2213,7 @@
     </row>
     <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>0</v>
@@ -2231,7 +2225,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>31</v>
@@ -2243,7 +2237,7 @@
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5" s="31" t="s">
         <v>30</v>
@@ -2255,7 +2249,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>32</v>
@@ -2267,7 +2261,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B7" s="33" t="s">
         <v>33</v>
@@ -2279,7 +2273,7 @@
     </row>
     <row r="8" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B8" s="31" t="s">
         <v>34</v>
@@ -2291,13 +2285,13 @@
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="B9" s="20" t="s">
-        <v>172</v>
-      </c>
       <c r="C9" s="43" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
     </row>
   </sheetData>
@@ -2318,16 +2312,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="57" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="B1" s="57" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="C1" s="60" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="D1" s="60" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2335,13 +2329,13 @@
         <v>45224</v>
       </c>
       <c r="B2" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="C2" s="61" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="D2" s="61" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2349,10 +2343,10 @@
         <v>45224</v>
       </c>
       <c r="B3" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="C3" s="61" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2360,13 +2354,13 @@
         <v>45224</v>
       </c>
       <c r="B4" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="C4" s="61" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="D4" s="61" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2374,10 +2368,10 @@
         <v>45224</v>
       </c>
       <c r="B5" t="s">
+        <v>343</v>
+      </c>
+      <c r="C5" s="61" t="s">
         <v>347</v>
-      </c>
-      <c r="C5" s="61" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -2385,10 +2379,10 @@
         <v>45224</v>
       </c>
       <c r="B6" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="D6" s="62" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2396,13 +2390,13 @@
         <v>45224</v>
       </c>
       <c r="B7" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="C7" s="61" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="D7" s="61" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>
@@ -2424,7 +2418,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
@@ -2435,86 +2429,86 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="72">
-        <v>1.84</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="71">
-        <v>1.84</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="30">
+      <c r="C4" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" s="36" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="37" t="str">
         <f>IF(C4=0,"Permanece",IF(C4="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="72">
-        <v>2.4500000000000002</v>
+        <v>2.4300000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="71">
-        <v>2.46</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" s="29" t="s">
         <v>17</v>
@@ -2526,7 +2520,7 @@
     </row>
     <row r="10" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" s="36" t="s">
         <v>2</v>
@@ -2538,38 +2532,38 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="72">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="71">
-        <v>0.75</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C13" s="6"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B14" s="29" t="s">
         <v>18</v>
@@ -2581,7 +2575,7 @@
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B15" s="36" t="s">
         <v>12</v>
@@ -2593,38 +2587,38 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="71">
-        <v>2.31</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C17" s="71">
-        <v>2.31</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="C18" s="6"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B19" s="29" t="s">
         <v>19</v>
@@ -2636,7 +2630,7 @@
     </row>
     <row r="20" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B20" s="36" t="s">
         <v>15</v>
@@ -2648,7 +2642,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>20</v>
@@ -2659,7 +2653,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>21</v>
@@ -2670,7 +2664,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>22</v>
@@ -2681,7 +2675,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>23</v>
@@ -2692,7 +2686,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>24</v>
@@ -2703,7 +2697,7 @@
     </row>
     <row r="26" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>25</v>
@@ -2714,112 +2708,112 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>26</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B28" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="26" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30" s="8" t="s">
         <v>36</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>28</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="27" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B32" s="8" t="s">
         <v>37</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>29</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="27" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>38</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="149.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>251</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -2859,7 +2853,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
@@ -2870,10 +2864,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C2" s="71">
         <v>3.93</v>
@@ -2881,56 +2875,56 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C3" s="71">
-        <v>3.94</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="C5" s="30" t="str">
+        <v>84</v>
+      </c>
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Sube</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C7" s="71">
         <v>0.34</v>
@@ -2938,10 +2932,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C8" s="71">
         <v>0.34</v>
@@ -2949,21 +2943,21 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
@@ -2972,10 +2966,10 @@
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" s="29" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
@@ -2984,10 +2978,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C12" s="71">
         <v>1.83</v>
@@ -2995,56 +2989,56 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C13" s="71">
-        <v>1.85</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="C15" s="30" t="str">
+        <v>96</v>
+      </c>
+      <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C17" s="74">
         <v>0</v>
@@ -3052,10 +3046,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C18" s="75">
         <v>0</v>
@@ -3063,10 +3057,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C19" s="75">
         <v>0</v>
@@ -3074,10 +3068,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C20" s="75">
         <v>0</v>
@@ -3085,10 +3079,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C21" s="75">
         <v>0</v>
@@ -3096,10 +3090,10 @@
     </row>
     <row r="22" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C22" s="76">
         <v>0</v>
@@ -3107,90 +3101,90 @@
     </row>
     <row r="23" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="26" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C23" s="73" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="27" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="26" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="26" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -3268,7 +3262,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
@@ -3279,43 +3273,43 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C2" s="72">
-        <v>0.56000000000000005</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C3" s="71">
-        <v>0.56000000000000005</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
@@ -3324,10 +3318,10 @@
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
@@ -3336,39 +3330,39 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C7" s="72"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C8" s="71"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
@@ -3377,10 +3371,10 @@
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" s="36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
@@ -3389,92 +3383,92 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="26" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C12" s="72">
-        <v>1.5</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C13" s="71">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C14" s="6"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16" s="36" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C17" s="71"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C18" s="71"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C19" s="6"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C20" s="30">
         <f>IFERROR(ROUND(ABS(C17-C18)*100,0),"-")</f>
@@ -3483,10 +3477,10 @@
     </row>
     <row r="21" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B21" s="36" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C21" s="37" t="str">
         <f>IFERROR(IF(C20=0,"Permanece",IF(SIGN(C20)=1,"Sube","Baja")),"-")</f>
@@ -3495,10 +3489,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C22" s="74">
         <v>0</v>
@@ -3506,10 +3500,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C23" s="75">
         <v>0</v>
@@ -3517,10 +3511,10 @@
     </row>
     <row r="24" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C24" s="76">
         <v>0</v>
@@ -3528,10 +3522,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C25" s="75">
         <v>0</v>
@@ -3539,10 +3533,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C26" s="75">
         <v>0</v>
@@ -3550,10 +3544,10 @@
     </row>
     <row r="27" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C27" s="76">
         <v>0</v>
@@ -3561,152 +3555,152 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="27" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="C34" s="9"/>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="25" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C35" s="10"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="26" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="27" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="26" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="27" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="165.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -3745,7 +3739,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
@@ -3756,10 +3750,10 @@
     </row>
     <row r="2" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="26" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C2" s="72">
         <v>0.45</v>
@@ -3767,10 +3761,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C3" s="72">
         <v>0.45</v>
@@ -3778,21 +3772,21 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
@@ -3801,10 +3795,10 @@
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
@@ -3813,10 +3807,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C7" s="74">
         <v>0</v>
@@ -3824,10 +3818,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="C8" s="75">
         <v>0</v>
@@ -3835,10 +3829,10 @@
     </row>
     <row r="9" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="C9" s="76">
         <v>0</v>
@@ -3846,10 +3840,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="C10" s="75">
         <v>0</v>
@@ -3857,10 +3851,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="C11" s="75">
         <v>0</v>
@@ -3868,10 +3862,10 @@
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="C12" s="76">
         <v>0</v>
@@ -3879,46 +3873,46 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="25" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -3958,7 +3952,7 @@
   <sheetData>
     <row r="1" spans="1:4" s="4" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
@@ -3969,68 +3963,68 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C2" s="72">
-        <v>2.4</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C3" s="71">
-        <v>2.42</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>208</v>
-      </c>
-      <c r="C5" s="30" t="str">
+        <v>207</v>
+      </c>
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D5" s="55"/>
     </row>
     <row r="6" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C7" s="72">
         <v>2.21</v>
@@ -4038,10 +4032,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C8" s="71">
         <v>2.21</v>
@@ -4049,21 +4043,21 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C10" s="30">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
@@ -4073,10 +4067,10 @@
     </row>
     <row r="11" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" s="36" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
@@ -4085,43 +4079,43 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C12" s="72">
-        <v>2.39</v>
+        <v>3.11</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C13" s="71">
-        <v>2.2400000000000002</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C15" s="30">
         <f>IF((C12-C13)&gt;=0,ROUND((C12-C13)*100,0),"")</f>
@@ -4130,10 +4124,10 @@
     </row>
     <row r="16" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16" s="29" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C16" s="37" t="str">
         <f>IF(C15=0,"Permanece",IF(C15="","Baja","Sube"))</f>
@@ -4142,100 +4136,100 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C17" s="72">
-        <v>1.32</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C18" s="71">
-        <v>1.27</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B20" s="29" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C20" s="30">
         <f>IF((C17-C18)&gt;=0,ROUND((C17-C18)*100,0),"")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B21" s="36" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C21" s="37" t="str">
         <f>IF(C20=0,"Permanece",IF(C20="","Baja","Sube"))</f>
-        <v>Sube</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C22" s="72">
-        <v>1.43</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C23" s="71">
-        <v>1.45</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B25" s="29" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C25" s="30" t="str">
         <f>IF((C22-C23)&gt;=0,ROUND((C22-C23)*100,0),"")</f>
@@ -4245,10 +4239,10 @@
     </row>
     <row r="26" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B26" s="36" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C26" s="37" t="str">
         <f>IF(C25=0,"Permanece",IF(C25="","Baja","Sube"))</f>
@@ -4258,113 +4252,111 @@
     </row>
     <row r="27" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="25" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="26" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C29" s="10"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>419</v>
-      </c>
+        <v>197</v>
+      </c>
+      <c r="C30" s="9"/>
     </row>
     <row r="31" spans="1:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C31" s="10"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="26" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="27" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C33" s="10"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="26" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C34" s="9"/>
     </row>
     <row r="35" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="27" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C35" s="10"/>
     </row>
     <row r="36" spans="1:3" ht="215.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -4403,7 +4395,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
@@ -4414,10 +4406,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C2" s="72">
         <v>9.56</v>
@@ -4425,67 +4417,67 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C3" s="71">
-        <v>9.57</v>
+        <v>9.56</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>227</v>
-      </c>
-      <c r="C5" s="30" t="str">
+        <v>226</v>
+      </c>
+      <c r="C5" s="30">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
-        <v>Baja</v>
+        <v>Permanece</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C7" s="72">
-        <v>1.92</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C8" s="71">
         <v>1.92</v>
@@ -4493,119 +4485,117 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="29" t="s">
-        <v>233</v>
-      </c>
-      <c r="C10" s="30">
+        <v>232</v>
+      </c>
+      <c r="C10" s="30" t="str">
         <f>IF((C7-C8)&gt;=0,ROUND((C7-C8)*100,0),"")</f>
-        <v>0</v>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B11" s="36" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C11" s="37" t="str">
         <f>IF(C10=0,"Permanece",IF(C10="","Baja","Sube"))</f>
-        <v>Permanece</v>
+        <v>Baja</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>237</v>
-      </c>
       <c r="C13" s="6" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C14" s="9"/>
     </row>
     <row r="15" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="27" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C15" s="10"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>403</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="C16" s="9"/>
     </row>
     <row r="17" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="27" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C17" s="10"/>
     </row>
     <row r="18" spans="1:3" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -4644,7 +4634,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>9</v>
@@ -4655,43 +4645,43 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="C2" s="72">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C3" s="71">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="C5" s="30" t="str">
         <f>IF((C2-C3)&gt;=0,ROUND((C2-C3)*100,0),"")</f>
@@ -4700,10 +4690,10 @@
     </row>
     <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="C6" s="37" t="str">
         <f>IF(C5=0,"Permanece",IF(C5="","Baja","Sube"))</f>
@@ -4712,10 +4702,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C7" s="74">
         <v>0</v>
@@ -4723,10 +4713,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="C8" s="75">
         <v>0</v>
@@ -4734,10 +4724,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C9" s="75">
         <v>0</v>
@@ -4745,10 +4735,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C10" s="75">
         <v>0</v>
@@ -4756,10 +4746,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C11" s="75">
         <v>0</v>
@@ -4767,10 +4757,10 @@
     </row>
     <row r="12" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="C12" s="76">
         <v>0</v>
@@ -4778,44 +4768,44 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="27" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="C14" s="10"/>
     </row>
     <row r="15" spans="1:3" ht="116.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>384</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="28" t="s">
-        <v>66</v>
-      </c>
       <c r="B16" s="12" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>365</v>
+        <v>431</v>
       </c>
     </row>
   </sheetData>
@@ -4863,10 +4853,10 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C1" s="44" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D1" s="49"/>
       <c r="E1" s="49"/>
@@ -4881,29 +4871,29 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
+        <v>430</v>
+      </c>
+      <c r="C2" s="47" t="s">
+        <v>264</v>
+      </c>
+      <c r="D2" s="47" t="s">
+        <v>261</v>
+      </c>
+      <c r="E2" s="47" t="s">
+        <v>262</v>
+      </c>
+      <c r="F2" s="48" t="s">
         <v>251</v>
-      </c>
-      <c r="C2" s="47" t="s">
-        <v>268</v>
-      </c>
-      <c r="D2" s="47" t="s">
-        <v>265</v>
-      </c>
-      <c r="E2" s="47" t="s">
-        <v>266</v>
-      </c>
-      <c r="F2" s="48" t="s">
-        <v>255</v>
       </c>
       <c r="G2" s="54"/>
       <c r="H2" s="54"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="45" t="s">
-        <v>365</v>
+        <v>431</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="D3" s="45">
         <v>70</v>
@@ -4912,24 +4902,24 @@
         <v>200</v>
       </c>
       <c r="F3" s="45" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="I3" s="45" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="J3" s="45" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="K3" s="45" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="45" t="s">
-        <v>252</v>
+        <v>432</v>
       </c>
       <c r="C4" s="45" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="D4" s="45">
         <v>30</v>
@@ -4938,31 +4928,23 @@
         <v>100</v>
       </c>
       <c r="F4" s="45" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="45" t="s">
-        <v>253</v>
+        <v>433</v>
       </c>
       <c r="F5" s="45" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="45" t="s">
-        <v>254</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="45" t="s">
-        <v>40</v>
-      </c>
       <c r="E7" s="47" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="F7" s="46" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="G7" s="46"/>
       <c r="H7" s="46"/>
@@ -4974,49 +4956,49 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E8" s="45" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="F8" s="45" t="s">
+        <v>299</v>
+      </c>
+      <c r="I8" s="45" t="s">
         <v>303</v>
       </c>
-      <c r="I8" s="45" t="s">
-        <v>307</v>
-      </c>
       <c r="J8" s="45" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E9" s="45" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="I9" s="45" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="J9" s="45" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E10" s="45" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="I10" s="45" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="C12" s="47" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="D12" s="47" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E12" s="47" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="F12" s="46" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="G12" s="46"/>
       <c r="H12" s="46"/>
@@ -5028,43 +5010,43 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D13" s="45" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="F13" s="45" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="I13" s="45" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D14" s="45" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="I14" s="45" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D15" s="45" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="I15" s="45" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="47" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="D17" s="47" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E17" s="47" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="F17" s="46" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="G17" s="46"/>
       <c r="H17" s="46"/>
@@ -5076,57 +5058,57 @@
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="F18" s="45" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="I18" s="45" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="F19" s="45" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="I19" s="45" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="50" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E22" s="50" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="F22" s="50" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="G22" s="50"/>
       <c r="H22" s="50"/>
       <c r="I22" s="50" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="J22" s="50" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="K22" s="50" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="L22" s="69" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
     </row>
     <row r="23" spans="3:13" s="63" customFormat="1" ht="99" x14ac:dyDescent="0.25">
       <c r="C23" s="63" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="D23" s="63" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E23" s="63" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="F23" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(YI!C21:C23)&gt;$D$3,SUM(YI!C21:C23)&gt;$E$3),$F$3,IF(OR(MAX(YI!C21:C23)&gt;$D$4,SUM(YI!C21:C23)&gt;$E$4),$F$4,$F$5)),D23,$I$3,SUM(YI!C21:C23),$J$3,MAX(YI!C21:C23),$K$3)</f>
@@ -5153,13 +5135,13 @@
     </row>
     <row r="24" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
       <c r="C24" s="51" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="D24" s="51" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="E24" s="51" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="F24" s="53" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$3,SUM(CUAREIM!C17:C19)&gt;$E$3),$F$3,IF(OR(MAX(CUAREIM!C17:C19)&gt;$D$4,SUM(CUAREIM!C17:C19)&gt;$E$4),$F$4,$F$5)),D24,$I$3,SUM(CUAREIM!C17:C19),$J$3,MAX(CUAREIM!C17:C19),$K$3)</f>
@@ -5169,7 +5151,7 @@
       <c r="H24" s="53"/>
       <c r="I24" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D24,IF(CUAREIM!C16=$E$8,$I$8,IF(CUAREIM!C16=$E$9,$I$9,$I$10)),$J$8,E24,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Cuareim se mantiene constante en la ciudad de Artigas. </v>
       </c>
       <c r="J24" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(CUAREIM!C27&gt;CUAREIM!C12,I13, IF(CUAREIM!C27=CUAREIM!C12,I14, I15)))</f>
@@ -5181,18 +5163,18 @@
       </c>
       <c r="L24" s="52" t="str">
         <f t="shared" ref="L24:L30" si="0">+_xlfn.CONCAT(F24," ",I24, " ",J24," ",K24)</f>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Cuareim está en descenso en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Cuareim, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Cuareim se mantiene constante en la ciudad de Artigas.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  </v>
       </c>
     </row>
     <row r="25" spans="3:13" ht="99" x14ac:dyDescent="0.3">
       <c r="C25" s="51" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="E25" s="51" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="F25" s="52" t="str">
         <f>_xlfn.CONCAT(IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$3,SUM(SANTALUCIA!C22:C24)&gt;$E$3),$F$3,IF(OR(MAX(SANTALUCIA!C22:C24)&gt;$D$4,SUM(SANTALUCIA!C22:C24)&gt;$E$4),$F$4,$F$5)),D25,$I$3,SUM(SANTALUCIA!C22:C24),$J$3,MAX(SANTALUCIA!C22:C24),$K$3)</f>
@@ -5202,7 +5184,7 @@
       <c r="H25" s="52"/>
       <c r="I25" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D25,IF(SANTALUCIA!C16=$E$8,$I$8,IF(SANTALUCIA!C16=$E$9,$I$9,$I$10)),$J$8,E25,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía. </v>
+        <v xml:space="preserve">Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía. </v>
       </c>
       <c r="J25" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(SANTALUCIA!C36&gt;SANTALUCIA!C12,I13, IF(SANTALUCIA!C36=SANTALUCIA!C12,I14, I15)))</f>
@@ -5214,18 +5196,18 @@
       </c>
       <c r="L25" s="52" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Santa Lucía está en ascenso en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
+        <v xml:space="preserve">En las últimas horas se registraron bajos acumulados de precipitación en la cuenca del río Santa Lucía, donde en las últimas 72 horas se acumularon 0 mm y con un máximo de 0 mm/día. Actualmente, el nivel del río Santa Lucía se mantiene constante en la ciudad de Santa Lucía.  Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días.  Existe una alta probabilidad de que el nivel supere al máximo registrado los días anteriores ( metros). </v>
       </c>
     </row>
     <row r="26" spans="3:13" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C26" s="51" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D26" s="51" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E26" s="51" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="F26" s="77" t="e">
         <f>_xlfn.CONCAT(IF(OR(MAX(URUGUAY!#REF!)&gt;$D$3,SUM(URUGUAY!#REF!)&gt;$E$3),$F$3,IF(OR(MAX(URUGUAY!#REF!)&gt;$D$4,SUM(URUGUAY!#REF!)&gt;$E$4),$F$4,$F$5)),D26,$I$3,SUM(URUGUAY!#REF!),$J$3,MAX(URUGUAY!#REF!),$K$3)</f>
@@ -5233,7 +5215,7 @@
       </c>
       <c r="I26" s="64" t="str">
         <f>IF(AND(URUGUAY!$C$11=$E$8,URUGUAY!$C$16=$E$8,URUGUAY!$C$21=$E$8,URUGUAY!$C$26=$E$8),_xlfn.CONCAT($F$8,$D$26,$I$8,$J$9," ",E26,", ",E27,", ",E28," y ",Tablas!E29,"."),IF(AND(URUGUAY!$C$11=$E$9,URUGUAY!$C$16=$E$9,URUGUAY!$C$21=$E$9,URUGUAY!$C$26=$E$9),_xlfn.CONCAT($F$8,$D$26,$I$9,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),IF(AND(URUGUAY!$C$11=$E$10,URUGUAY!$C$16=$E$10,URUGUAY!$C$21=$E$10,URUGUAY!$C$26=$E$10),_xlfn.CONCAT($F$8,$D$26,$I$10,$J$9," ",E26,", ",E27,", ",E28," y ",E29,"."),_xlfn.CONCAT($F$8,D26,I27,I28,I29))))</f>
-        <v>Actualmente, el nivel del río Uruguay está en ascenso en las ciudades de Salto Paysandú; se mantiene constante en la ciudad de  Bella Unión; está en descenso en la ciudad de  Fray Bentos.</v>
+        <v>Actualmente, el nivel del río Uruguay está en ascenso en la ciudad de  Salto; se mantiene constante en las ciudades de Bella Unión Paysandú; está en descenso en la ciudad de  Fray Bentos.</v>
       </c>
       <c r="J26" s="78" t="str">
         <f>_xlfn.CONCAT(F13,IF(AND(URUGUAY!C28&gt;URUGUAY!C7, URUGUAY!C30&gt;URUGUAY!C12, URUGUAY!C32&gt;URUGUAY!C17, URUGUAY!C34&gt;URUGUAY!C22),I13, IF(AND(URUGUAY!C28=URUGUAY!C7, URUGUAY!C30=URUGUAY!C12, URUGUAY!C32=URUGUAY!C17, URUGUAY!C34=URUGUAY!C22),I14, I15)))</f>
@@ -5248,24 +5230,24 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="27" spans="3:13" ht="33" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C27" s="51"/>
       <c r="D27" s="51"/>
       <c r="E27" s="51" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="F27" s="77"/>
       <c r="G27" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E8, URUGUAY!$C$16=Tablas!E8,URUGUAY!$C$21=Tablas!E8,URUGUAY!$C$26=Tablas!E8)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E8,_xlfn.CONCAT(" ",$E$26,),""),IF(URUGUAY!$C$16=Tablas!E8,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E8,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E8,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Salto Paysandú</v>
+        <v xml:space="preserve"> Salto</v>
       </c>
       <c r="I27" s="65" t="str">
         <f>_xlfn.CONCAT(I8,IF(G27&gt;1,$J$9,$J$8),H27, IF(G27=4,".", ";"))</f>
-        <v xml:space="preserve"> está en ascenso en las ciudades de Salto Paysandú;</v>
+        <v xml:space="preserve"> está en ascenso en la ciudad de  Salto;</v>
       </c>
       <c r="J27" s="78"/>
       <c r="K27" s="78"/>
@@ -5275,20 +5257,20 @@
       <c r="C28" s="51"/>
       <c r="D28" s="51"/>
       <c r="E28" s="51" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="F28" s="77"/>
       <c r="G28" s="58">
         <f>SUM(URUGUAY!$C$11=Tablas!E9, URUGUAY!$C$16=Tablas!E9,URUGUAY!$C$21=Tablas!E9,URUGUAY!$C$26=Tablas!E9)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28" s="59" t="str">
         <f>_xlfn.CONCAT(IF(URUGUAY!$C$11=Tablas!E9,_xlfn.CONCAT(" ",$E$26),""),IF(URUGUAY!$C$16=Tablas!E9,_xlfn.CONCAT(" ",$E$27),""),IF(URUGUAY!$C$21=Tablas!E9,_xlfn.CONCAT(" ",$E$28),""),IF(URUGUAY!$C$26=Tablas!E9,_xlfn.CONCAT(" ",$E$29),""))</f>
-        <v xml:space="preserve"> Bella Unión</v>
+        <v xml:space="preserve"> Bella Unión Paysandú</v>
       </c>
       <c r="I28" s="65" t="str">
         <f>_xlfn.CONCAT(I9,IF(G28&gt;1,$J$9,$J$8),H28, IF((G27+G28)=4,".", ";"))</f>
-        <v xml:space="preserve"> se mantiene constante en la ciudad de  Bella Unión;</v>
+        <v xml:space="preserve"> se mantiene constante en las ciudades de Bella Unión Paysandú;</v>
       </c>
       <c r="J28" s="78"/>
       <c r="K28" s="78"/>
@@ -5298,7 +5280,7 @@
       <c r="C29" s="51"/>
       <c r="D29" s="51"/>
       <c r="E29" s="51" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="F29" s="77"/>
       <c r="G29" s="58">
@@ -5317,15 +5299,15 @@
       <c r="K29" s="78"/>
       <c r="L29" s="78"/>
     </row>
-    <row r="30" spans="3:13" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:13" ht="66" x14ac:dyDescent="0.3">
       <c r="C30" s="51" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="D30" s="51" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="E30" s="51" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="F30" s="52" t="e">
         <f>_xlfn.CONCAT(IF(OR(MAX(NEGRO!#REF!)&gt;$D$3,SUM(NEGRO!#REF!)&gt;$E$3),$F$3,IF(OR(MAX(NEGRO!#REF!)&gt;$D$4,SUM(NEGRO!#REF!)&gt;$E$4),$F$4,$F$5)),D30,$I$3,SUM(NEGRO!#REF!),$J$3,MAX(NEGRO!#REF!),$K$3)</f>
@@ -5335,11 +5317,11 @@
       <c r="H30" s="52"/>
       <c r="I30" s="64" t="str">
         <f>_xlfn.CONCAT($F$8,D30,IF(NEGRO!C11=$E$8,$I$8,IF(NEGRO!C11=$E$9,$I$9,$I$10)),$J$8,E30,". ")</f>
-        <v xml:space="preserve">Actualmente, el nivel del Río Negro se mantiene constante en la ciudad de Mercedes. </v>
+        <v xml:space="preserve">Actualmente, el nivel del Río Negro está en descenso en la ciudad de Mercedes. </v>
       </c>
       <c r="J30" s="53" t="str">
         <f>_xlfn.CONCAT(F13,IF(NEGRO!C16&gt;NEGRO!C7,I13, IF(NEGRO!C16=NEGRO!C7,I14, I15)))</f>
-        <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, existe la posibilidad de nuevos incrementos de nivel en los próximos días. </v>
+        <v xml:space="preserve">Considerando las lluvias pronosticadas y los niveles registrados en las estaciones de monitoreo, se prevé que el nivel descienda en los próximos días. </v>
       </c>
       <c r="K30" s="66" t="str">
         <f>IF(NEGRO!C9="-","",IF(NEGRO!C16&gt;NEGRO!C9,_xlfn.CONCAT(F18,NEGRO!C9,I18),_xlfn.CONCAT(F19,NEGRO!C9,I19)))</f>

</xml_diff>